<commit_message>
them cot chia gang CR trong file excel
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF5EEF1-CA57-49DA-9953-B5DE697C19A0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF5EE9C-14A2-41BD-B6BC-7C8A92B27B8F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
   <si>
     <t>STT</t>
   </si>
@@ -138,7 +138,10 @@
     <t>KR</t>
   </si>
   <si>
-    <t>KL gang chia (T)</t>
+    <t>KL gang chia CCT(T)</t>
+  </si>
+  <si>
+    <t>KL gang chia CR(T)</t>
   </si>
 </sst>
 </file>
@@ -704,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:AT29"/>
+  <dimension ref="A1:AU29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -729,21 +732,21 @@
     <col min="22" max="22" width="33.28515625" style="1" customWidth="1"/>
     <col min="23" max="23" width="12" style="1" customWidth="1"/>
     <col min="24" max="24" width="9.7109375" style="1" customWidth="1"/>
-    <col min="25" max="26" width="9.42578125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="10.42578125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.140625" style="1"/>
-    <col min="30" max="31" width="10.7109375" style="1" customWidth="1"/>
-    <col min="32" max="33" width="10.85546875" style="1" customWidth="1"/>
-    <col min="34" max="35" width="19.28515625" style="1" customWidth="1"/>
-    <col min="36" max="36" width="19.5703125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="9.140625" style="1"/>
-    <col min="38" max="38" width="25.5703125" style="1" customWidth="1"/>
-    <col min="39" max="39" width="17.140625" style="1" customWidth="1"/>
-    <col min="40" max="16384" width="9.140625" style="1"/>
+    <col min="25" max="27" width="9.42578125" style="1" customWidth="1"/>
+    <col min="28" max="28" width="10.42578125" style="1" customWidth="1"/>
+    <col min="29" max="29" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="9.140625" style="1"/>
+    <col min="31" max="32" width="10.7109375" style="1" customWidth="1"/>
+    <col min="33" max="34" width="10.85546875" style="1" customWidth="1"/>
+    <col min="35" max="36" width="19.28515625" style="1" customWidth="1"/>
+    <col min="37" max="37" width="19.5703125" style="1" customWidth="1"/>
+    <col min="38" max="38" width="9.140625" style="1"/>
+    <col min="39" max="39" width="25.5703125" style="1" customWidth="1"/>
+    <col min="40" max="40" width="17.140625" style="1" customWidth="1"/>
+    <col min="41" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -752,7 +755,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:46" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:47" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -761,7 +764,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:46" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:47" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -803,8 +806,9 @@
       <c r="AK4" s="19"/>
       <c r="AL4" s="19"/>
       <c r="AM4" s="19"/>
-    </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
+      <c r="AN4" s="19"/>
+    </row>
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -844,8 +848,9 @@
       <c r="AK5" s="17"/>
       <c r="AL5" s="17"/>
       <c r="AM5" s="17"/>
-    </row>
-    <row r="7" spans="1:46" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AN5" s="17"/>
+    </row>
+    <row r="7" spans="1:47" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -925,46 +930,49 @@
         <v>37</v>
       </c>
       <c r="AA7" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AB7" s="10" t="s">
+      <c r="AC7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AC7" s="10" t="s">
+      <c r="AD7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AD7" s="10" t="s">
+      <c r="AE7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AE7" s="10" t="s">
+      <c r="AF7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AG7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AG7" s="10" t="s">
+      <c r="AH7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="AH7" s="10" t="s">
+      <c r="AI7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="AI7" s="10" t="s">
+      <c r="AJ7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AJ7" s="11" t="s">
+      <c r="AK7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AK7" s="12" t="s">
+      <c r="AL7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AL7" s="12" t="s">
+      <c r="AM7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AM7" s="12" t="s">
+      <c r="AN7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:46" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:47" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -1000,19 +1008,20 @@
       <c r="AG8" s="13"/>
       <c r="AH8" s="13"/>
       <c r="AI8" s="13"/>
-      <c r="AJ8" s="15"/>
+      <c r="AJ8" s="13"/>
       <c r="AK8" s="15"/>
       <c r="AL8" s="15"/>
       <c r="AM8" s="15"/>
-      <c r="AN8" s="5"/>
+      <c r="AN8" s="15"/>
       <c r="AO8" s="5"/>
       <c r="AP8" s="5"/>
       <c r="AQ8" s="5"/>
       <c r="AR8" s="5"/>
       <c r="AS8" s="5"/>
       <c r="AT8" s="5"/>
-    </row>
-    <row r="9" spans="1:46" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AU8" s="5"/>
+    </row>
+    <row r="9" spans="1:47" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1059,8 +1068,9 @@
       <c r="AR9" s="5"/>
       <c r="AS9" s="5"/>
       <c r="AT9" s="5"/>
-    </row>
-    <row r="10" spans="1:46" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AU9" s="5"/>
+    </row>
+    <row r="10" spans="1:47" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1107,8 +1117,9 @@
       <c r="AR10" s="5"/>
       <c r="AS10" s="5"/>
       <c r="AT10" s="5"/>
-    </row>
-    <row r="11" spans="1:46" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AU10" s="5"/>
+    </row>
+    <row r="11" spans="1:47" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1155,8 +1166,9 @@
       <c r="AR11" s="5"/>
       <c r="AS11" s="5"/>
       <c r="AT11" s="5"/>
-    </row>
-    <row r="12" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU11" s="5"/>
+    </row>
+    <row r="12" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1203,8 +1215,9 @@
       <c r="AR12" s="5"/>
       <c r="AS12" s="5"/>
       <c r="AT12" s="5"/>
-    </row>
-    <row r="13" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU12" s="5"/>
+    </row>
+    <row r="13" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1251,8 +1264,9 @@
       <c r="AR13" s="5"/>
       <c r="AS13" s="5"/>
       <c r="AT13" s="5"/>
-    </row>
-    <row r="14" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU13" s="5"/>
+    </row>
+    <row r="14" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1299,8 +1313,9 @@
       <c r="AR14" s="5"/>
       <c r="AS14" s="5"/>
       <c r="AT14" s="5"/>
-    </row>
-    <row r="15" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU14" s="5"/>
+    </row>
+    <row r="15" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1347,8 +1362,9 @@
       <c r="AR15" s="5"/>
       <c r="AS15" s="5"/>
       <c r="AT15" s="5"/>
-    </row>
-    <row r="16" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU15" s="5"/>
+    </row>
+    <row r="16" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1395,8 +1411,9 @@
       <c r="AR16" s="5"/>
       <c r="AS16" s="5"/>
       <c r="AT16" s="5"/>
-    </row>
-    <row r="17" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU16" s="5"/>
+    </row>
+    <row r="17" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1443,8 +1460,9 @@
       <c r="AR17" s="5"/>
       <c r="AS17" s="5"/>
       <c r="AT17" s="5"/>
-    </row>
-    <row r="18" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU17" s="5"/>
+    </row>
+    <row r="18" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1491,8 +1509,9 @@
       <c r="AR18" s="5"/>
       <c r="AS18" s="5"/>
       <c r="AT18" s="5"/>
-    </row>
-    <row r="19" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU18" s="5"/>
+    </row>
+    <row r="19" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1539,8 +1558,9 @@
       <c r="AR19" s="5"/>
       <c r="AS19" s="5"/>
       <c r="AT19" s="5"/>
-    </row>
-    <row r="20" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU19" s="5"/>
+    </row>
+    <row r="20" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1587,8 +1607,9 @@
       <c r="AR20" s="5"/>
       <c r="AS20" s="5"/>
       <c r="AT20" s="5"/>
-    </row>
-    <row r="21" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU20" s="5"/>
+    </row>
+    <row r="21" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1635,8 +1656,9 @@
       <c r="AR21" s="5"/>
       <c r="AS21" s="5"/>
       <c r="AT21" s="5"/>
-    </row>
-    <row r="22" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU21" s="5"/>
+    </row>
+    <row r="22" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1683,8 +1705,9 @@
       <c r="AR22" s="5"/>
       <c r="AS22" s="5"/>
       <c r="AT22" s="5"/>
-    </row>
-    <row r="23" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU22" s="5"/>
+    </row>
+    <row r="23" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1731,8 +1754,9 @@
       <c r="AR23" s="5"/>
       <c r="AS23" s="5"/>
       <c r="AT23" s="5"/>
-    </row>
-    <row r="24" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU23" s="5"/>
+    </row>
+    <row r="24" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1779,8 +1803,9 @@
       <c r="AR24" s="5"/>
       <c r="AS24" s="5"/>
       <c r="AT24" s="5"/>
-    </row>
-    <row r="25" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU24" s="5"/>
+    </row>
+    <row r="25" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1827,8 +1852,9 @@
       <c r="AR25" s="5"/>
       <c r="AS25" s="5"/>
       <c r="AT25" s="5"/>
-    </row>
-    <row r="26" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU25" s="5"/>
+    </row>
+    <row r="26" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1875,8 +1901,9 @@
       <c r="AR26" s="5"/>
       <c r="AS26" s="5"/>
       <c r="AT26" s="5"/>
-    </row>
-    <row r="27" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU26" s="5"/>
+    </row>
+    <row r="27" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1923,8 +1950,9 @@
       <c r="AR27" s="5"/>
       <c r="AS27" s="5"/>
       <c r="AT27" s="5"/>
-    </row>
-    <row r="28" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU27" s="5"/>
+    </row>
+    <row r="28" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1971,8 +1999,9 @@
       <c r="AR28" s="5"/>
       <c r="AS28" s="5"/>
       <c r="AT28" s="5"/>
-    </row>
-    <row r="29" spans="1:46" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AU28" s="5"/>
+    </row>
+    <row r="29" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2019,12 +2048,13 @@
       <c r="AR29" s="5"/>
       <c r="AS29" s="5"/>
       <c r="AT29" s="5"/>
+      <c r="AU29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AM5"/>
+    <mergeCell ref="A5:AN5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AM4"/>
+    <mergeCell ref="A4:AN4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
them cot san ra gang
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF5EE9C-14A2-41BD-B6BC-7C8A92B27B8F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268C8168-3DB7-43C3-8E40-3288A82E2303}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>STT</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t>KL gang chia CR(T)</t>
+  </si>
+  <si>
+    <t>Sàn ra gang</t>
   </si>
 </sst>
 </file>
@@ -707,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:AU29"/>
+  <dimension ref="A1:AV29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -719,34 +722,34 @@
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.42578125" style="1" customWidth="1"/>
-    <col min="10" max="11" width="12.42578125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" style="1" customWidth="1"/>
-    <col min="13" max="14" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.85546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="10.42578125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="8.5703125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="33.28515625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="12" style="1" customWidth="1"/>
-    <col min="24" max="24" width="9.7109375" style="1" customWidth="1"/>
-    <col min="25" max="27" width="9.42578125" style="1" customWidth="1"/>
-    <col min="28" max="28" width="10.42578125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="9.140625" style="1"/>
-    <col min="31" max="32" width="10.7109375" style="1" customWidth="1"/>
-    <col min="33" max="34" width="10.85546875" style="1" customWidth="1"/>
-    <col min="35" max="36" width="19.28515625" style="1" customWidth="1"/>
-    <col min="37" max="37" width="19.5703125" style="1" customWidth="1"/>
-    <col min="38" max="38" width="9.140625" style="1"/>
-    <col min="39" max="39" width="25.5703125" style="1" customWidth="1"/>
-    <col min="40" max="40" width="17.140625" style="1" customWidth="1"/>
-    <col min="41" max="16384" width="9.140625" style="1"/>
+    <col min="10" max="12" width="12.42578125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.42578125" style="1" customWidth="1"/>
+    <col min="14" max="15" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.85546875" style="1" customWidth="1"/>
+    <col min="18" max="18" width="10.42578125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="16.85546875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.5703125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="33.28515625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="12" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.7109375" style="1" customWidth="1"/>
+    <col min="26" max="28" width="9.42578125" style="1" customWidth="1"/>
+    <col min="29" max="29" width="10.42578125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.140625" style="1"/>
+    <col min="32" max="33" width="10.7109375" style="1" customWidth="1"/>
+    <col min="34" max="35" width="10.85546875" style="1" customWidth="1"/>
+    <col min="36" max="37" width="19.28515625" style="1" customWidth="1"/>
+    <col min="38" max="38" width="19.5703125" style="1" customWidth="1"/>
+    <col min="39" max="39" width="9.140625" style="1"/>
+    <col min="40" max="40" width="25.5703125" style="1" customWidth="1"/>
+    <col min="41" max="41" width="17.140625" style="1" customWidth="1"/>
+    <col min="42" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:48" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -755,7 +758,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:47" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:48" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -764,7 +767,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:47" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:48" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -807,8 +810,9 @@
       <c r="AL4" s="19"/>
       <c r="AM4" s="19"/>
       <c r="AN4" s="19"/>
-    </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AO4" s="19"/>
+    </row>
+    <row r="5" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -849,8 +853,9 @@
       <c r="AL5" s="17"/>
       <c r="AM5" s="17"/>
       <c r="AN5" s="17"/>
-    </row>
-    <row r="7" spans="1:47" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AO5" s="17"/>
+    </row>
+    <row r="7" spans="1:48" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -884,95 +889,98 @@
       <c r="K7" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="Q7" s="9" t="s">
+      <c r="R7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="R7" s="9" t="s">
+      <c r="S7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="S7" s="10" t="s">
+      <c r="T7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="T7" s="10" t="s">
+      <c r="U7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="U7" s="10" t="s">
+      <c r="V7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="V7" s="10" t="s">
+      <c r="W7" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="W7" s="10" t="s">
+      <c r="X7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="X7" s="10" t="s">
+      <c r="Y7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="Y7" s="10" t="s">
+      <c r="Z7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="Z7" s="10" t="s">
+      <c r="AA7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AA7" s="10" t="s">
+      <c r="AB7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="AB7" s="10" t="s">
+      <c r="AC7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AC7" s="10" t="s">
+      <c r="AD7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AD7" s="10" t="s">
+      <c r="AE7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AE7" s="10" t="s">
+      <c r="AF7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AG7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AG7" s="10" t="s">
+      <c r="AH7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AH7" s="10" t="s">
+      <c r="AI7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="AI7" s="10" t="s">
+      <c r="AJ7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="AJ7" s="10" t="s">
+      <c r="AK7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AK7" s="11" t="s">
+      <c r="AL7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AL7" s="12" t="s">
+      <c r="AM7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AM7" s="12" t="s">
+      <c r="AN7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AN7" s="12" t="s">
+      <c r="AO7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:47" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:48" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -984,14 +992,14 @@
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
-      <c r="L8" s="15"/>
+      <c r="L8" s="14"/>
       <c r="M8" s="15"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="16"/>
       <c r="R8" s="15"/>
-      <c r="S8" s="13"/>
+      <c r="S8" s="15"/>
       <c r="T8" s="13"/>
       <c r="U8" s="13"/>
       <c r="V8" s="13"/>
@@ -1009,19 +1017,20 @@
       <c r="AH8" s="13"/>
       <c r="AI8" s="13"/>
       <c r="AJ8" s="13"/>
-      <c r="AK8" s="15"/>
+      <c r="AK8" s="13"/>
       <c r="AL8" s="15"/>
       <c r="AM8" s="15"/>
       <c r="AN8" s="15"/>
-      <c r="AO8" s="5"/>
+      <c r="AO8" s="15"/>
       <c r="AP8" s="5"/>
       <c r="AQ8" s="5"/>
       <c r="AR8" s="5"/>
       <c r="AS8" s="5"/>
       <c r="AT8" s="5"/>
       <c r="AU8" s="5"/>
-    </row>
-    <row r="9" spans="1:47" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AV8" s="5"/>
+    </row>
+    <row r="9" spans="1:48" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1038,8 +1047,8 @@
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
       <c r="P9" s="6"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="5"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="7"/>
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
@@ -1069,8 +1078,9 @@
       <c r="AS9" s="5"/>
       <c r="AT9" s="5"/>
       <c r="AU9" s="5"/>
-    </row>
-    <row r="10" spans="1:47" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AV9" s="5"/>
+    </row>
+    <row r="10" spans="1:48" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1087,8 +1097,8 @@
       <c r="N10" s="6"/>
       <c r="O10" s="6"/>
       <c r="P10" s="6"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="5"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="7"/>
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
@@ -1118,8 +1128,9 @@
       <c r="AS10" s="5"/>
       <c r="AT10" s="5"/>
       <c r="AU10" s="5"/>
-    </row>
-    <row r="11" spans="1:47" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AV10" s="5"/>
+    </row>
+    <row r="11" spans="1:48" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1136,8 +1147,8 @@
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="5"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="7"/>
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
@@ -1167,8 +1178,9 @@
       <c r="AS11" s="5"/>
       <c r="AT11" s="5"/>
       <c r="AU11" s="5"/>
-    </row>
-    <row r="12" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV11" s="5"/>
+    </row>
+    <row r="12" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1216,8 +1228,9 @@
       <c r="AS12" s="5"/>
       <c r="AT12" s="5"/>
       <c r="AU12" s="5"/>
-    </row>
-    <row r="13" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV12" s="5"/>
+    </row>
+    <row r="13" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1265,8 +1278,9 @@
       <c r="AS13" s="5"/>
       <c r="AT13" s="5"/>
       <c r="AU13" s="5"/>
-    </row>
-    <row r="14" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV13" s="5"/>
+    </row>
+    <row r="14" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1314,8 +1328,9 @@
       <c r="AS14" s="5"/>
       <c r="AT14" s="5"/>
       <c r="AU14" s="5"/>
-    </row>
-    <row r="15" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV14" s="5"/>
+    </row>
+    <row r="15" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1363,8 +1378,9 @@
       <c r="AS15" s="5"/>
       <c r="AT15" s="5"/>
       <c r="AU15" s="5"/>
-    </row>
-    <row r="16" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV15" s="5"/>
+    </row>
+    <row r="16" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1412,8 +1428,9 @@
       <c r="AS16" s="5"/>
       <c r="AT16" s="5"/>
       <c r="AU16" s="5"/>
-    </row>
-    <row r="17" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV16" s="5"/>
+    </row>
+    <row r="17" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1461,8 +1478,9 @@
       <c r="AS17" s="5"/>
       <c r="AT17" s="5"/>
       <c r="AU17" s="5"/>
-    </row>
-    <row r="18" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV17" s="5"/>
+    </row>
+    <row r="18" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1510,8 +1528,9 @@
       <c r="AS18" s="5"/>
       <c r="AT18" s="5"/>
       <c r="AU18" s="5"/>
-    </row>
-    <row r="19" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV18" s="5"/>
+    </row>
+    <row r="19" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1559,8 +1578,9 @@
       <c r="AS19" s="5"/>
       <c r="AT19" s="5"/>
       <c r="AU19" s="5"/>
-    </row>
-    <row r="20" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV19" s="5"/>
+    </row>
+    <row r="20" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1608,8 +1628,9 @@
       <c r="AS20" s="5"/>
       <c r="AT20" s="5"/>
       <c r="AU20" s="5"/>
-    </row>
-    <row r="21" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV20" s="5"/>
+    </row>
+    <row r="21" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1657,8 +1678,9 @@
       <c r="AS21" s="5"/>
       <c r="AT21" s="5"/>
       <c r="AU21" s="5"/>
-    </row>
-    <row r="22" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV21" s="5"/>
+    </row>
+    <row r="22" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1706,8 +1728,9 @@
       <c r="AS22" s="5"/>
       <c r="AT22" s="5"/>
       <c r="AU22" s="5"/>
-    </row>
-    <row r="23" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV22" s="5"/>
+    </row>
+    <row r="23" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1755,8 +1778,9 @@
       <c r="AS23" s="5"/>
       <c r="AT23" s="5"/>
       <c r="AU23" s="5"/>
-    </row>
-    <row r="24" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV23" s="5"/>
+    </row>
+    <row r="24" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1804,8 +1828,9 @@
       <c r="AS24" s="5"/>
       <c r="AT24" s="5"/>
       <c r="AU24" s="5"/>
-    </row>
-    <row r="25" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV24" s="5"/>
+    </row>
+    <row r="25" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1853,8 +1878,9 @@
       <c r="AS25" s="5"/>
       <c r="AT25" s="5"/>
       <c r="AU25" s="5"/>
-    </row>
-    <row r="26" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV25" s="5"/>
+    </row>
+    <row r="26" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1902,8 +1928,9 @@
       <c r="AS26" s="5"/>
       <c r="AT26" s="5"/>
       <c r="AU26" s="5"/>
-    </row>
-    <row r="27" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV26" s="5"/>
+    </row>
+    <row r="27" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1951,8 +1978,9 @@
       <c r="AS27" s="5"/>
       <c r="AT27" s="5"/>
       <c r="AU27" s="5"/>
-    </row>
-    <row r="28" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV27" s="5"/>
+    </row>
+    <row r="28" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2000,8 +2028,9 @@
       <c r="AS28" s="5"/>
       <c r="AT28" s="5"/>
       <c r="AU28" s="5"/>
-    </row>
-    <row r="29" spans="1:47" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AV28" s="5"/>
+    </row>
+    <row r="29" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2049,12 +2078,13 @@
       <c r="AS29" s="5"/>
       <c r="AT29" s="5"/>
       <c r="AU29" s="5"/>
+      <c r="AV29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AN5"/>
+    <mergeCell ref="A5:AO5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AN4"/>
+    <mergeCell ref="A4:AO4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
them cot tinh trang QLCL form thong ke
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268C8168-3DB7-43C3-8E40-3288A82E2303}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F41B7D-178D-4EC2-9616-BCBAE8A6D910}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t>STT</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>Sàn ra gang</t>
+  </si>
+  <si>
+    <t>Tình trạng QLCL</t>
   </si>
 </sst>
 </file>
@@ -710,7 +713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:AV29"/>
+  <dimension ref="A1:AW29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -722,34 +725,35 @@
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.42578125" style="1" customWidth="1"/>
-    <col min="10" max="12" width="12.42578125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="9.42578125" style="1" customWidth="1"/>
-    <col min="14" max="15" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.85546875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="10.42578125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="16.85546875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.5703125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="33.28515625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="12" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.7109375" style="1" customWidth="1"/>
-    <col min="26" max="28" width="9.42578125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="10.42578125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="9.140625" style="1"/>
-    <col min="32" max="33" width="10.7109375" style="1" customWidth="1"/>
-    <col min="34" max="35" width="10.85546875" style="1" customWidth="1"/>
-    <col min="36" max="37" width="19.28515625" style="1" customWidth="1"/>
-    <col min="38" max="38" width="19.5703125" style="1" customWidth="1"/>
-    <col min="39" max="39" width="9.140625" style="1"/>
-    <col min="40" max="40" width="25.5703125" style="1" customWidth="1"/>
-    <col min="41" max="41" width="17.140625" style="1" customWidth="1"/>
-    <col min="42" max="16384" width="9.140625" style="1"/>
+    <col min="10" max="10" width="19.85546875" style="1" customWidth="1"/>
+    <col min="11" max="13" width="12.42578125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" style="1" customWidth="1"/>
+    <col min="15" max="16" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.85546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="10.42578125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="16.85546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="8.5703125" style="1" customWidth="1"/>
+    <col min="22" max="22" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="33.28515625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="12" style="1" customWidth="1"/>
+    <col min="26" max="26" width="9.7109375" style="1" customWidth="1"/>
+    <col min="27" max="29" width="9.42578125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="10.42578125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="9.140625" style="1"/>
+    <col min="33" max="34" width="10.7109375" style="1" customWidth="1"/>
+    <col min="35" max="36" width="10.85546875" style="1" customWidth="1"/>
+    <col min="37" max="38" width="19.28515625" style="1" customWidth="1"/>
+    <col min="39" max="39" width="19.5703125" style="1" customWidth="1"/>
+    <col min="40" max="40" width="12.7109375" style="1" customWidth="1"/>
+    <col min="41" max="41" width="25.5703125" style="1" customWidth="1"/>
+    <col min="42" max="42" width="17.140625" style="1" customWidth="1"/>
+    <col min="43" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -758,7 +762,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:48" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -767,7 +771,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:48" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:49" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -811,8 +815,9 @@
       <c r="AM4" s="19"/>
       <c r="AN4" s="19"/>
       <c r="AO4" s="19"/>
-    </row>
-    <row r="5" spans="1:48" x14ac:dyDescent="0.25">
+      <c r="AP4" s="19"/>
+    </row>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -854,8 +859,9 @@
       <c r="AM5" s="17"/>
       <c r="AN5" s="17"/>
       <c r="AO5" s="17"/>
-    </row>
-    <row r="7" spans="1:48" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AP5" s="17"/>
+    </row>
+    <row r="7" spans="1:49" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -883,104 +889,107 @@
       <c r="I7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="M7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="R7" s="9" t="s">
+      <c r="S7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="S7" s="9" t="s">
+      <c r="T7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="10" t="s">
+      <c r="U7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="U7" s="10" t="s">
+      <c r="V7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="V7" s="10" t="s">
+      <c r="W7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="W7" s="10" t="s">
+      <c r="X7" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="X7" s="10" t="s">
+      <c r="Y7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="Y7" s="10" t="s">
+      <c r="Z7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="Z7" s="10" t="s">
+      <c r="AA7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="AA7" s="10" t="s">
+      <c r="AB7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AB7" s="10" t="s">
+      <c r="AC7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="AC7" s="10" t="s">
+      <c r="AD7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AD7" s="10" t="s">
+      <c r="AE7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AE7" s="10" t="s">
+      <c r="AF7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AG7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AG7" s="10" t="s">
+      <c r="AH7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AH7" s="10" t="s">
+      <c r="AI7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AI7" s="10" t="s">
+      <c r="AJ7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="AJ7" s="10" t="s">
+      <c r="AK7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="AK7" s="10" t="s">
+      <c r="AL7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AL7" s="11" t="s">
+      <c r="AM7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AM7" s="12" t="s">
+      <c r="AN7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AN7" s="12" t="s">
+      <c r="AO7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AO7" s="12" t="s">
+      <c r="AP7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:48" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -993,14 +1002,14 @@
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
       <c r="L8" s="14"/>
-      <c r="M8" s="15"/>
+      <c r="M8" s="14"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
       <c r="P8" s="15"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="15"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="16"/>
       <c r="S8" s="15"/>
-      <c r="T8" s="13"/>
+      <c r="T8" s="15"/>
       <c r="U8" s="13"/>
       <c r="V8" s="13"/>
       <c r="W8" s="13"/>
@@ -1018,19 +1027,20 @@
       <c r="AI8" s="13"/>
       <c r="AJ8" s="13"/>
       <c r="AK8" s="13"/>
-      <c r="AL8" s="15"/>
+      <c r="AL8" s="13"/>
       <c r="AM8" s="15"/>
       <c r="AN8" s="15"/>
       <c r="AO8" s="15"/>
-      <c r="AP8" s="5"/>
+      <c r="AP8" s="15"/>
       <c r="AQ8" s="5"/>
       <c r="AR8" s="5"/>
       <c r="AS8" s="5"/>
       <c r="AT8" s="5"/>
       <c r="AU8" s="5"/>
       <c r="AV8" s="5"/>
-    </row>
-    <row r="9" spans="1:48" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AW8" s="5"/>
+    </row>
+    <row r="9" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1048,8 +1058,8 @@
       <c r="O9" s="6"/>
       <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
-      <c r="R9" s="7"/>
-      <c r="S9" s="5"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="7"/>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
       <c r="V9" s="5"/>
@@ -1079,8 +1089,9 @@
       <c r="AT9" s="5"/>
       <c r="AU9" s="5"/>
       <c r="AV9" s="5"/>
-    </row>
-    <row r="10" spans="1:48" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AW9" s="5"/>
+    </row>
+    <row r="10" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1098,8 +1109,8 @@
       <c r="O10" s="6"/>
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
-      <c r="R10" s="7"/>
-      <c r="S10" s="5"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="7"/>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
       <c r="V10" s="5"/>
@@ -1129,8 +1140,9 @@
       <c r="AT10" s="5"/>
       <c r="AU10" s="5"/>
       <c r="AV10" s="5"/>
-    </row>
-    <row r="11" spans="1:48" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AW10" s="5"/>
+    </row>
+    <row r="11" spans="1:49" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1148,8 +1160,8 @@
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
-      <c r="R11" s="7"/>
-      <c r="S11" s="5"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="7"/>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
       <c r="V11" s="5"/>
@@ -1179,8 +1191,9 @@
       <c r="AT11" s="5"/>
       <c r="AU11" s="5"/>
       <c r="AV11" s="5"/>
-    </row>
-    <row r="12" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW11" s="5"/>
+    </row>
+    <row r="12" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1229,8 +1242,9 @@
       <c r="AT12" s="5"/>
       <c r="AU12" s="5"/>
       <c r="AV12" s="5"/>
-    </row>
-    <row r="13" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW12" s="5"/>
+    </row>
+    <row r="13" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1279,8 +1293,9 @@
       <c r="AT13" s="5"/>
       <c r="AU13" s="5"/>
       <c r="AV13" s="5"/>
-    </row>
-    <row r="14" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW13" s="5"/>
+    </row>
+    <row r="14" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1329,8 +1344,9 @@
       <c r="AT14" s="5"/>
       <c r="AU14" s="5"/>
       <c r="AV14" s="5"/>
-    </row>
-    <row r="15" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW14" s="5"/>
+    </row>
+    <row r="15" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1379,8 +1395,9 @@
       <c r="AT15" s="5"/>
       <c r="AU15" s="5"/>
       <c r="AV15" s="5"/>
-    </row>
-    <row r="16" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW15" s="5"/>
+    </row>
+    <row r="16" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1429,8 +1446,9 @@
       <c r="AT16" s="5"/>
       <c r="AU16" s="5"/>
       <c r="AV16" s="5"/>
-    </row>
-    <row r="17" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW16" s="5"/>
+    </row>
+    <row r="17" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1479,8 +1497,9 @@
       <c r="AT17" s="5"/>
       <c r="AU17" s="5"/>
       <c r="AV17" s="5"/>
-    </row>
-    <row r="18" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW17" s="5"/>
+    </row>
+    <row r="18" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1529,8 +1548,9 @@
       <c r="AT18" s="5"/>
       <c r="AU18" s="5"/>
       <c r="AV18" s="5"/>
-    </row>
-    <row r="19" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW18" s="5"/>
+    </row>
+    <row r="19" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1579,8 +1599,9 @@
       <c r="AT19" s="5"/>
       <c r="AU19" s="5"/>
       <c r="AV19" s="5"/>
-    </row>
-    <row r="20" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW19" s="5"/>
+    </row>
+    <row r="20" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1629,8 +1650,9 @@
       <c r="AT20" s="5"/>
       <c r="AU20" s="5"/>
       <c r="AV20" s="5"/>
-    </row>
-    <row r="21" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW20" s="5"/>
+    </row>
+    <row r="21" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1679,8 +1701,9 @@
       <c r="AT21" s="5"/>
       <c r="AU21" s="5"/>
       <c r="AV21" s="5"/>
-    </row>
-    <row r="22" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW21" s="5"/>
+    </row>
+    <row r="22" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1729,8 +1752,9 @@
       <c r="AT22" s="5"/>
       <c r="AU22" s="5"/>
       <c r="AV22" s="5"/>
-    </row>
-    <row r="23" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW22" s="5"/>
+    </row>
+    <row r="23" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1779,8 +1803,9 @@
       <c r="AT23" s="5"/>
       <c r="AU23" s="5"/>
       <c r="AV23" s="5"/>
-    </row>
-    <row r="24" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW23" s="5"/>
+    </row>
+    <row r="24" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1829,8 +1854,9 @@
       <c r="AT24" s="5"/>
       <c r="AU24" s="5"/>
       <c r="AV24" s="5"/>
-    </row>
-    <row r="25" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW24" s="5"/>
+    </row>
+    <row r="25" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1879,8 +1905,9 @@
       <c r="AT25" s="5"/>
       <c r="AU25" s="5"/>
       <c r="AV25" s="5"/>
-    </row>
-    <row r="26" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW25" s="5"/>
+    </row>
+    <row r="26" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1929,8 +1956,9 @@
       <c r="AT26" s="5"/>
       <c r="AU26" s="5"/>
       <c r="AV26" s="5"/>
-    </row>
-    <row r="27" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW26" s="5"/>
+    </row>
+    <row r="27" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -1979,8 +2007,9 @@
       <c r="AT27" s="5"/>
       <c r="AU27" s="5"/>
       <c r="AV27" s="5"/>
-    </row>
-    <row r="28" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW27" s="5"/>
+    </row>
+    <row r="28" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2029,8 +2058,9 @@
       <c r="AT28" s="5"/>
       <c r="AU28" s="5"/>
       <c r="AV28" s="5"/>
-    </row>
-    <row r="29" spans="1:48" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AW28" s="5"/>
+    </row>
+    <row r="29" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2079,12 +2109,13 @@
       <c r="AT29" s="5"/>
       <c r="AU29" s="5"/>
       <c r="AV29" s="5"/>
+      <c r="AW29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AO5"/>
+    <mergeCell ref="A5:AP5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AO4"/>
+    <mergeCell ref="A4:AP4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
them cot nhiet do
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F41B7D-178D-4EC2-9616-BCBAE8A6D910}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CB3DD1-E2DE-4E40-BAD0-CF6EBBE8D179}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t>STT</t>
   </si>
@@ -148,6 +148,10 @@
   </si>
   <si>
     <t>Tình trạng QLCL</t>
+  </si>
+  <si>
+    <t>Nhiệt độ
+(ºC)</t>
   </si>
 </sst>
 </file>
@@ -713,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:AW29"/>
+  <dimension ref="A1:AX29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -737,23 +741,24 @@
     <col min="22" max="22" width="7" style="1" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="33.28515625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="12" style="1" customWidth="1"/>
-    <col min="26" max="26" width="9.7109375" style="1" customWidth="1"/>
-    <col min="27" max="29" width="9.42578125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="10.42578125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.140625" style="1"/>
-    <col min="33" max="34" width="10.7109375" style="1" customWidth="1"/>
-    <col min="35" max="36" width="10.85546875" style="1" customWidth="1"/>
-    <col min="37" max="38" width="19.28515625" style="1" customWidth="1"/>
-    <col min="39" max="39" width="19.5703125" style="1" customWidth="1"/>
-    <col min="40" max="40" width="12.7109375" style="1" customWidth="1"/>
-    <col min="41" max="41" width="25.5703125" style="1" customWidth="1"/>
-    <col min="42" max="42" width="17.140625" style="1" customWidth="1"/>
-    <col min="43" max="16384" width="9.140625" style="1"/>
+    <col min="25" max="25" width="14.7109375" style="1" customWidth="1"/>
+    <col min="26" max="26" width="12" style="1" customWidth="1"/>
+    <col min="27" max="27" width="9.7109375" style="1" customWidth="1"/>
+    <col min="28" max="30" width="9.42578125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="10.42578125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.140625" style="1"/>
+    <col min="34" max="35" width="10.7109375" style="1" customWidth="1"/>
+    <col min="36" max="37" width="10.85546875" style="1" customWidth="1"/>
+    <col min="38" max="39" width="19.28515625" style="1" customWidth="1"/>
+    <col min="40" max="40" width="19.5703125" style="1" customWidth="1"/>
+    <col min="41" max="41" width="12.7109375" style="1" customWidth="1"/>
+    <col min="42" max="42" width="25.5703125" style="1" customWidth="1"/>
+    <col min="43" max="43" width="17.140625" style="1" customWidth="1"/>
+    <col min="44" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:50" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -762,7 +767,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:49" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:50" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -771,7 +776,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:49" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:50" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -816,8 +821,9 @@
       <c r="AN4" s="19"/>
       <c r="AO4" s="19"/>
       <c r="AP4" s="19"/>
-    </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="AQ4" s="19"/>
+    </row>
+    <row r="5" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -860,8 +866,9 @@
       <c r="AN5" s="17"/>
       <c r="AO5" s="17"/>
       <c r="AP5" s="17"/>
-    </row>
-    <row r="7" spans="1:49" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AQ5" s="17"/>
+    </row>
+    <row r="7" spans="1:50" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -935,61 +942,64 @@
         <v>1</v>
       </c>
       <c r="Y7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="Z7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="Z7" s="10" t="s">
+      <c r="AA7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AA7" s="10" t="s">
+      <c r="AB7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="AB7" s="10" t="s">
+      <c r="AC7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AC7" s="10" t="s">
+      <c r="AD7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="AD7" s="10" t="s">
+      <c r="AE7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AE7" s="10" t="s">
+      <c r="AF7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AG7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AG7" s="10" t="s">
+      <c r="AH7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AH7" s="10" t="s">
+      <c r="AI7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AI7" s="10" t="s">
+      <c r="AJ7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AJ7" s="10" t="s">
+      <c r="AK7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="AK7" s="10" t="s">
+      <c r="AL7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="AL7" s="10" t="s">
+      <c r="AM7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AM7" s="11" t="s">
+      <c r="AN7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AN7" s="12" t="s">
+      <c r="AO7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AO7" s="12" t="s">
+      <c r="AP7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AP7" s="12" t="s">
+      <c r="AQ7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:50" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -1028,19 +1038,20 @@
       <c r="AJ8" s="13"/>
       <c r="AK8" s="13"/>
       <c r="AL8" s="13"/>
-      <c r="AM8" s="15"/>
+      <c r="AM8" s="13"/>
       <c r="AN8" s="15"/>
       <c r="AO8" s="15"/>
       <c r="AP8" s="15"/>
-      <c r="AQ8" s="5"/>
+      <c r="AQ8" s="15"/>
       <c r="AR8" s="5"/>
       <c r="AS8" s="5"/>
       <c r="AT8" s="5"/>
       <c r="AU8" s="5"/>
       <c r="AV8" s="5"/>
       <c r="AW8" s="5"/>
-    </row>
-    <row r="9" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AX8" s="5"/>
+    </row>
+    <row r="9" spans="1:50" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1090,8 +1101,9 @@
       <c r="AU9" s="5"/>
       <c r="AV9" s="5"/>
       <c r="AW9" s="5"/>
-    </row>
-    <row r="10" spans="1:49" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AX9" s="5"/>
+    </row>
+    <row r="10" spans="1:50" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1141,8 +1153,9 @@
       <c r="AU10" s="5"/>
       <c r="AV10" s="5"/>
       <c r="AW10" s="5"/>
-    </row>
-    <row r="11" spans="1:49" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AX10" s="5"/>
+    </row>
+    <row r="11" spans="1:50" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1192,8 +1205,9 @@
       <c r="AU11" s="5"/>
       <c r="AV11" s="5"/>
       <c r="AW11" s="5"/>
-    </row>
-    <row r="12" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX11" s="5"/>
+    </row>
+    <row r="12" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1243,8 +1257,9 @@
       <c r="AU12" s="5"/>
       <c r="AV12" s="5"/>
       <c r="AW12" s="5"/>
-    </row>
-    <row r="13" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX12" s="5"/>
+    </row>
+    <row r="13" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1294,8 +1309,9 @@
       <c r="AU13" s="5"/>
       <c r="AV13" s="5"/>
       <c r="AW13" s="5"/>
-    </row>
-    <row r="14" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX13" s="5"/>
+    </row>
+    <row r="14" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1345,8 +1361,9 @@
       <c r="AU14" s="5"/>
       <c r="AV14" s="5"/>
       <c r="AW14" s="5"/>
-    </row>
-    <row r="15" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX14" s="5"/>
+    </row>
+    <row r="15" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1396,8 +1413,9 @@
       <c r="AU15" s="5"/>
       <c r="AV15" s="5"/>
       <c r="AW15" s="5"/>
-    </row>
-    <row r="16" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX15" s="5"/>
+    </row>
+    <row r="16" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1447,8 +1465,9 @@
       <c r="AU16" s="5"/>
       <c r="AV16" s="5"/>
       <c r="AW16" s="5"/>
-    </row>
-    <row r="17" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX16" s="5"/>
+    </row>
+    <row r="17" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1498,8 +1517,9 @@
       <c r="AU17" s="5"/>
       <c r="AV17" s="5"/>
       <c r="AW17" s="5"/>
-    </row>
-    <row r="18" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX17" s="5"/>
+    </row>
+    <row r="18" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1549,8 +1569,9 @@
       <c r="AU18" s="5"/>
       <c r="AV18" s="5"/>
       <c r="AW18" s="5"/>
-    </row>
-    <row r="19" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX18" s="5"/>
+    </row>
+    <row r="19" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1600,8 +1621,9 @@
       <c r="AU19" s="5"/>
       <c r="AV19" s="5"/>
       <c r="AW19" s="5"/>
-    </row>
-    <row r="20" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX19" s="5"/>
+    </row>
+    <row r="20" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1651,8 +1673,9 @@
       <c r="AU20" s="5"/>
       <c r="AV20" s="5"/>
       <c r="AW20" s="5"/>
-    </row>
-    <row r="21" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX20" s="5"/>
+    </row>
+    <row r="21" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1702,8 +1725,9 @@
       <c r="AU21" s="5"/>
       <c r="AV21" s="5"/>
       <c r="AW21" s="5"/>
-    </row>
-    <row r="22" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX21" s="5"/>
+    </row>
+    <row r="22" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1753,8 +1777,9 @@
       <c r="AU22" s="5"/>
       <c r="AV22" s="5"/>
       <c r="AW22" s="5"/>
-    </row>
-    <row r="23" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX22" s="5"/>
+    </row>
+    <row r="23" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1804,8 +1829,9 @@
       <c r="AU23" s="5"/>
       <c r="AV23" s="5"/>
       <c r="AW23" s="5"/>
-    </row>
-    <row r="24" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX23" s="5"/>
+    </row>
+    <row r="24" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1855,8 +1881,9 @@
       <c r="AU24" s="5"/>
       <c r="AV24" s="5"/>
       <c r="AW24" s="5"/>
-    </row>
-    <row r="25" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX24" s="5"/>
+    </row>
+    <row r="25" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1906,8 +1933,9 @@
       <c r="AU25" s="5"/>
       <c r="AV25" s="5"/>
       <c r="AW25" s="5"/>
-    </row>
-    <row r="26" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX25" s="5"/>
+    </row>
+    <row r="26" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1957,8 +1985,9 @@
       <c r="AU26" s="5"/>
       <c r="AV26" s="5"/>
       <c r="AW26" s="5"/>
-    </row>
-    <row r="27" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX26" s="5"/>
+    </row>
+    <row r="27" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2008,8 +2037,9 @@
       <c r="AU27" s="5"/>
       <c r="AV27" s="5"/>
       <c r="AW27" s="5"/>
-    </row>
-    <row r="28" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX27" s="5"/>
+    </row>
+    <row r="28" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2059,8 +2089,9 @@
       <c r="AU28" s="5"/>
       <c r="AV28" s="5"/>
       <c r="AW28" s="5"/>
-    </row>
-    <row r="29" spans="1:49" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AX28" s="5"/>
+    </row>
+    <row r="29" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2110,12 +2141,13 @@
       <c r="AU29" s="5"/>
       <c r="AV29" s="5"/>
       <c r="AW29" s="5"/>
+      <c r="AX29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AP5"/>
+    <mergeCell ref="A5:AQ5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AP4"/>
+    <mergeCell ref="A4:AQ4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
sua doi ten nhiet do
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CB3DD1-E2DE-4E40-BAD0-CF6EBBE8D179}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DAD426-DEB0-4472-B5DE-7A6740970DC3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -150,7 +150,7 @@
     <t>Tình trạng QLCL</t>
   </si>
   <si>
-    <t>Nhiệt độ
+    <t>Nhiệt độ trước khi rót
 (ºC)</t>
   </si>
 </sst>

</xml_diff>

<commit_message>
them cot kl thung va gang truoc KR
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DAD426-DEB0-4472-B5DE-7A6740970DC3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F5BB1E-8984-4D12-B7E7-553AD5FC61CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>STT</t>
   </si>
@@ -152,6 +152,9 @@
   <si>
     <t>Nhiệt độ trước khi rót
 (ºC)</t>
+  </si>
+  <si>
+    <t>KL Thùng và Gang trước KR (T)</t>
   </si>
 </sst>
 </file>
@@ -717,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:AX29"/>
+  <dimension ref="A1:AY29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -745,20 +748,21 @@
     <col min="26" max="26" width="12" style="1" customWidth="1"/>
     <col min="27" max="27" width="9.7109375" style="1" customWidth="1"/>
     <col min="28" max="30" width="9.42578125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="10.42578125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.140625" style="1"/>
-    <col min="34" max="35" width="10.7109375" style="1" customWidth="1"/>
-    <col min="36" max="37" width="10.85546875" style="1" customWidth="1"/>
-    <col min="38" max="39" width="19.28515625" style="1" customWidth="1"/>
-    <col min="40" max="40" width="19.5703125" style="1" customWidth="1"/>
-    <col min="41" max="41" width="12.7109375" style="1" customWidth="1"/>
-    <col min="42" max="42" width="25.5703125" style="1" customWidth="1"/>
-    <col min="43" max="43" width="17.140625" style="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="1"/>
+    <col min="31" max="31" width="12.42578125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="10.42578125" style="1" customWidth="1"/>
+    <col min="33" max="33" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.140625" style="1"/>
+    <col min="35" max="36" width="10.7109375" style="1" customWidth="1"/>
+    <col min="37" max="38" width="10.85546875" style="1" customWidth="1"/>
+    <col min="39" max="40" width="19.28515625" style="1" customWidth="1"/>
+    <col min="41" max="41" width="19.5703125" style="1" customWidth="1"/>
+    <col min="42" max="42" width="12.7109375" style="1" customWidth="1"/>
+    <col min="43" max="43" width="25.5703125" style="1" customWidth="1"/>
+    <col min="44" max="44" width="17.140625" style="1" customWidth="1"/>
+    <col min="45" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:51" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -767,7 +771,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:50" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:51" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -776,7 +780,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:50" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:51" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -822,8 +826,9 @@
       <c r="AO4" s="19"/>
       <c r="AP4" s="19"/>
       <c r="AQ4" s="19"/>
-    </row>
-    <row r="5" spans="1:50" x14ac:dyDescent="0.25">
+      <c r="AR4" s="19"/>
+    </row>
+    <row r="5" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -867,8 +872,9 @@
       <c r="AO5" s="17"/>
       <c r="AP5" s="17"/>
       <c r="AQ5" s="17"/>
-    </row>
-    <row r="7" spans="1:50" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AR5" s="17"/>
+    </row>
+    <row r="7" spans="1:51" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -960,46 +966,49 @@
         <v>38</v>
       </c>
       <c r="AE7" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AG7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AG7" s="10" t="s">
+      <c r="AH7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AH7" s="10" t="s">
+      <c r="AI7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AI7" s="10" t="s">
+      <c r="AJ7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AJ7" s="10" t="s">
+      <c r="AK7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AK7" s="10" t="s">
+      <c r="AL7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="AL7" s="10" t="s">
+      <c r="AM7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="AM7" s="10" t="s">
+      <c r="AN7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AN7" s="11" t="s">
+      <c r="AO7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AO7" s="12" t="s">
+      <c r="AP7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AP7" s="12" t="s">
+      <c r="AQ7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AQ7" s="12" t="s">
+      <c r="AR7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:50" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:51" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -1039,19 +1048,20 @@
       <c r="AK8" s="13"/>
       <c r="AL8" s="13"/>
       <c r="AM8" s="13"/>
-      <c r="AN8" s="15"/>
+      <c r="AN8" s="13"/>
       <c r="AO8" s="15"/>
       <c r="AP8" s="15"/>
       <c r="AQ8" s="15"/>
-      <c r="AR8" s="5"/>
+      <c r="AR8" s="15"/>
       <c r="AS8" s="5"/>
       <c r="AT8" s="5"/>
       <c r="AU8" s="5"/>
       <c r="AV8" s="5"/>
       <c r="AW8" s="5"/>
       <c r="AX8" s="5"/>
-    </row>
-    <row r="9" spans="1:50" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AY8" s="5"/>
+    </row>
+    <row r="9" spans="1:51" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1102,8 +1112,9 @@
       <c r="AV9" s="5"/>
       <c r="AW9" s="5"/>
       <c r="AX9" s="5"/>
-    </row>
-    <row r="10" spans="1:50" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AY9" s="5"/>
+    </row>
+    <row r="10" spans="1:51" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1154,8 +1165,9 @@
       <c r="AV10" s="5"/>
       <c r="AW10" s="5"/>
       <c r="AX10" s="5"/>
-    </row>
-    <row r="11" spans="1:50" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AY10" s="5"/>
+    </row>
+    <row r="11" spans="1:51" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1206,8 +1218,9 @@
       <c r="AV11" s="5"/>
       <c r="AW11" s="5"/>
       <c r="AX11" s="5"/>
-    </row>
-    <row r="12" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY11" s="5"/>
+    </row>
+    <row r="12" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1258,8 +1271,9 @@
       <c r="AV12" s="5"/>
       <c r="AW12" s="5"/>
       <c r="AX12" s="5"/>
-    </row>
-    <row r="13" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY12" s="5"/>
+    </row>
+    <row r="13" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1310,8 +1324,9 @@
       <c r="AV13" s="5"/>
       <c r="AW13" s="5"/>
       <c r="AX13" s="5"/>
-    </row>
-    <row r="14" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY13" s="5"/>
+    </row>
+    <row r="14" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1362,8 +1377,9 @@
       <c r="AV14" s="5"/>
       <c r="AW14" s="5"/>
       <c r="AX14" s="5"/>
-    </row>
-    <row r="15" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY14" s="5"/>
+    </row>
+    <row r="15" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1414,8 +1430,9 @@
       <c r="AV15" s="5"/>
       <c r="AW15" s="5"/>
       <c r="AX15" s="5"/>
-    </row>
-    <row r="16" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY15" s="5"/>
+    </row>
+    <row r="16" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1466,8 +1483,9 @@
       <c r="AV16" s="5"/>
       <c r="AW16" s="5"/>
       <c r="AX16" s="5"/>
-    </row>
-    <row r="17" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY16" s="5"/>
+    </row>
+    <row r="17" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1518,8 +1536,9 @@
       <c r="AV17" s="5"/>
       <c r="AW17" s="5"/>
       <c r="AX17" s="5"/>
-    </row>
-    <row r="18" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY17" s="5"/>
+    </row>
+    <row r="18" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1570,8 +1589,9 @@
       <c r="AV18" s="5"/>
       <c r="AW18" s="5"/>
       <c r="AX18" s="5"/>
-    </row>
-    <row r="19" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY18" s="5"/>
+    </row>
+    <row r="19" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1622,8 +1642,9 @@
       <c r="AV19" s="5"/>
       <c r="AW19" s="5"/>
       <c r="AX19" s="5"/>
-    </row>
-    <row r="20" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY19" s="5"/>
+    </row>
+    <row r="20" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1674,8 +1695,9 @@
       <c r="AV20" s="5"/>
       <c r="AW20" s="5"/>
       <c r="AX20" s="5"/>
-    </row>
-    <row r="21" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY20" s="5"/>
+    </row>
+    <row r="21" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1726,8 +1748,9 @@
       <c r="AV21" s="5"/>
       <c r="AW21" s="5"/>
       <c r="AX21" s="5"/>
-    </row>
-    <row r="22" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY21" s="5"/>
+    </row>
+    <row r="22" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1778,8 +1801,9 @@
       <c r="AV22" s="5"/>
       <c r="AW22" s="5"/>
       <c r="AX22" s="5"/>
-    </row>
-    <row r="23" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY22" s="5"/>
+    </row>
+    <row r="23" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1830,8 +1854,9 @@
       <c r="AV23" s="5"/>
       <c r="AW23" s="5"/>
       <c r="AX23" s="5"/>
-    </row>
-    <row r="24" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY23" s="5"/>
+    </row>
+    <row r="24" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1882,8 +1907,9 @@
       <c r="AV24" s="5"/>
       <c r="AW24" s="5"/>
       <c r="AX24" s="5"/>
-    </row>
-    <row r="25" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY24" s="5"/>
+    </row>
+    <row r="25" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1934,8 +1960,9 @@
       <c r="AV25" s="5"/>
       <c r="AW25" s="5"/>
       <c r="AX25" s="5"/>
-    </row>
-    <row r="26" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY25" s="5"/>
+    </row>
+    <row r="26" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -1986,8 +2013,9 @@
       <c r="AV26" s="5"/>
       <c r="AW26" s="5"/>
       <c r="AX26" s="5"/>
-    </row>
-    <row r="27" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY26" s="5"/>
+    </row>
+    <row r="27" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2038,8 +2066,9 @@
       <c r="AV27" s="5"/>
       <c r="AW27" s="5"/>
       <c r="AX27" s="5"/>
-    </row>
-    <row r="28" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY27" s="5"/>
+    </row>
+    <row r="28" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2090,8 +2119,9 @@
       <c r="AV28" s="5"/>
       <c r="AW28" s="5"/>
       <c r="AX28" s="5"/>
-    </row>
-    <row r="29" spans="1:50" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AY28" s="5"/>
+    </row>
+    <row r="29" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2142,12 +2172,13 @@
       <c r="AV29" s="5"/>
       <c r="AW29" s="5"/>
       <c r="AX29" s="5"/>
+      <c r="AY29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AQ5"/>
+    <mergeCell ref="A5:AR5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AQ4"/>
+    <mergeCell ref="A4:AR4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
phan bo KL Xi
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F5BB1E-8984-4D12-B7E7-553AD5FC61CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8F736E-6AF6-4FAB-A2A8-66CFF2EE5BBD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
   <si>
     <t>STT</t>
   </si>
@@ -155,6 +155,15 @@
   </si>
   <si>
     <t>KL Thùng và Gang trước KR (T)</t>
+  </si>
+  <si>
+    <t>KL xỉ KR (T)</t>
+  </si>
+  <si>
+    <t>KL chia xỉ KR (T)</t>
+  </si>
+  <si>
+    <t>KL gang CCT + Xỉ (T)</t>
   </si>
 </sst>
 </file>
@@ -720,7 +729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:AY29"/>
+  <dimension ref="A1:BB29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -755,14 +764,17 @@
     <col min="35" max="36" width="10.7109375" style="1" customWidth="1"/>
     <col min="37" max="38" width="10.85546875" style="1" customWidth="1"/>
     <col min="39" max="40" width="19.28515625" style="1" customWidth="1"/>
-    <col min="41" max="41" width="19.5703125" style="1" customWidth="1"/>
-    <col min="42" max="42" width="12.7109375" style="1" customWidth="1"/>
-    <col min="43" max="43" width="25.5703125" style="1" customWidth="1"/>
-    <col min="44" max="44" width="17.140625" style="1" customWidth="1"/>
-    <col min="45" max="16384" width="9.140625" style="1"/>
+    <col min="41" max="41" width="15.140625" style="1" customWidth="1"/>
+    <col min="42" max="42" width="12.28515625" style="1" customWidth="1"/>
+    <col min="43" max="43" width="13.140625" style="1" customWidth="1"/>
+    <col min="44" max="44" width="19.5703125" style="1" customWidth="1"/>
+    <col min="45" max="45" width="12.7109375" style="1" customWidth="1"/>
+    <col min="46" max="46" width="25.5703125" style="1" customWidth="1"/>
+    <col min="47" max="47" width="17.140625" style="1" customWidth="1"/>
+    <col min="48" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:54" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -771,7 +783,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:51" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:54" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -780,7 +792,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:51" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:54" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -827,8 +839,11 @@
       <c r="AP4" s="19"/>
       <c r="AQ4" s="19"/>
       <c r="AR4" s="19"/>
-    </row>
-    <row r="5" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="AS4" s="19"/>
+      <c r="AT4" s="19"/>
+      <c r="AU4" s="19"/>
+    </row>
+    <row r="5" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -873,8 +888,11 @@
       <c r="AP5" s="17"/>
       <c r="AQ5" s="17"/>
       <c r="AR5" s="17"/>
-    </row>
-    <row r="7" spans="1:51" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS5" s="17"/>
+      <c r="AT5" s="17"/>
+      <c r="AU5" s="17"/>
+    </row>
+    <row r="7" spans="1:54" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -995,20 +1013,29 @@
       <c r="AN7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AO7" s="11" t="s">
+      <c r="AO7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="AP7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AQ7" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="AR7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AP7" s="12" t="s">
+      <c r="AS7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AQ7" s="12" t="s">
+      <c r="AT7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AR7" s="12" t="s">
+      <c r="AU7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:51" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -1049,19 +1076,22 @@
       <c r="AL8" s="13"/>
       <c r="AM8" s="13"/>
       <c r="AN8" s="13"/>
-      <c r="AO8" s="15"/>
-      <c r="AP8" s="15"/>
-      <c r="AQ8" s="15"/>
+      <c r="AO8" s="13"/>
+      <c r="AP8" s="13"/>
+      <c r="AQ8" s="13"/>
       <c r="AR8" s="15"/>
-      <c r="AS8" s="5"/>
-      <c r="AT8" s="5"/>
-      <c r="AU8" s="5"/>
+      <c r="AS8" s="15"/>
+      <c r="AT8" s="15"/>
+      <c r="AU8" s="15"/>
       <c r="AV8" s="5"/>
       <c r="AW8" s="5"/>
       <c r="AX8" s="5"/>
       <c r="AY8" s="5"/>
-    </row>
-    <row r="9" spans="1:51" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AZ8" s="5"/>
+      <c r="BA8" s="5"/>
+      <c r="BB8" s="5"/>
+    </row>
+    <row r="9" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1113,8 +1143,11 @@
       <c r="AW9" s="5"/>
       <c r="AX9" s="5"/>
       <c r="AY9" s="5"/>
-    </row>
-    <row r="10" spans="1:51" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AZ9" s="5"/>
+      <c r="BA9" s="5"/>
+      <c r="BB9" s="5"/>
+    </row>
+    <row r="10" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1166,8 +1199,11 @@
       <c r="AW10" s="5"/>
       <c r="AX10" s="5"/>
       <c r="AY10" s="5"/>
-    </row>
-    <row r="11" spans="1:51" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AZ10" s="5"/>
+      <c r="BA10" s="5"/>
+      <c r="BB10" s="5"/>
+    </row>
+    <row r="11" spans="1:54" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1219,8 +1255,11 @@
       <c r="AW11" s="5"/>
       <c r="AX11" s="5"/>
       <c r="AY11" s="5"/>
-    </row>
-    <row r="12" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ11" s="5"/>
+      <c r="BA11" s="5"/>
+      <c r="BB11" s="5"/>
+    </row>
+    <row r="12" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1272,8 +1311,11 @@
       <c r="AW12" s="5"/>
       <c r="AX12" s="5"/>
       <c r="AY12" s="5"/>
-    </row>
-    <row r="13" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ12" s="5"/>
+      <c r="BA12" s="5"/>
+      <c r="BB12" s="5"/>
+    </row>
+    <row r="13" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1325,8 +1367,11 @@
       <c r="AW13" s="5"/>
       <c r="AX13" s="5"/>
       <c r="AY13" s="5"/>
-    </row>
-    <row r="14" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ13" s="5"/>
+      <c r="BA13" s="5"/>
+      <c r="BB13" s="5"/>
+    </row>
+    <row r="14" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1378,8 +1423,11 @@
       <c r="AW14" s="5"/>
       <c r="AX14" s="5"/>
       <c r="AY14" s="5"/>
-    </row>
-    <row r="15" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ14" s="5"/>
+      <c r="BA14" s="5"/>
+      <c r="BB14" s="5"/>
+    </row>
+    <row r="15" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1431,8 +1479,11 @@
       <c r="AW15" s="5"/>
       <c r="AX15" s="5"/>
       <c r="AY15" s="5"/>
-    </row>
-    <row r="16" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ15" s="5"/>
+      <c r="BA15" s="5"/>
+      <c r="BB15" s="5"/>
+    </row>
+    <row r="16" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1484,8 +1535,11 @@
       <c r="AW16" s="5"/>
       <c r="AX16" s="5"/>
       <c r="AY16" s="5"/>
-    </row>
-    <row r="17" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ16" s="5"/>
+      <c r="BA16" s="5"/>
+      <c r="BB16" s="5"/>
+    </row>
+    <row r="17" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1537,8 +1591,11 @@
       <c r="AW17" s="5"/>
       <c r="AX17" s="5"/>
       <c r="AY17" s="5"/>
-    </row>
-    <row r="18" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ17" s="5"/>
+      <c r="BA17" s="5"/>
+      <c r="BB17" s="5"/>
+    </row>
+    <row r="18" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1590,8 +1647,11 @@
       <c r="AW18" s="5"/>
       <c r="AX18" s="5"/>
       <c r="AY18" s="5"/>
-    </row>
-    <row r="19" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ18" s="5"/>
+      <c r="BA18" s="5"/>
+      <c r="BB18" s="5"/>
+    </row>
+    <row r="19" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1643,8 +1703,11 @@
       <c r="AW19" s="5"/>
       <c r="AX19" s="5"/>
       <c r="AY19" s="5"/>
-    </row>
-    <row r="20" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ19" s="5"/>
+      <c r="BA19" s="5"/>
+      <c r="BB19" s="5"/>
+    </row>
+    <row r="20" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1696,8 +1759,11 @@
       <c r="AW20" s="5"/>
       <c r="AX20" s="5"/>
       <c r="AY20" s="5"/>
-    </row>
-    <row r="21" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ20" s="5"/>
+      <c r="BA20" s="5"/>
+      <c r="BB20" s="5"/>
+    </row>
+    <row r="21" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1749,8 +1815,11 @@
       <c r="AW21" s="5"/>
       <c r="AX21" s="5"/>
       <c r="AY21" s="5"/>
-    </row>
-    <row r="22" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ21" s="5"/>
+      <c r="BA21" s="5"/>
+      <c r="BB21" s="5"/>
+    </row>
+    <row r="22" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1802,8 +1871,11 @@
       <c r="AW22" s="5"/>
       <c r="AX22" s="5"/>
       <c r="AY22" s="5"/>
-    </row>
-    <row r="23" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ22" s="5"/>
+      <c r="BA22" s="5"/>
+      <c r="BB22" s="5"/>
+    </row>
+    <row r="23" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1855,8 +1927,11 @@
       <c r="AW23" s="5"/>
       <c r="AX23" s="5"/>
       <c r="AY23" s="5"/>
-    </row>
-    <row r="24" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ23" s="5"/>
+      <c r="BA23" s="5"/>
+      <c r="BB23" s="5"/>
+    </row>
+    <row r="24" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1908,8 +1983,11 @@
       <c r="AW24" s="5"/>
       <c r="AX24" s="5"/>
       <c r="AY24" s="5"/>
-    </row>
-    <row r="25" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ24" s="5"/>
+      <c r="BA24" s="5"/>
+      <c r="BB24" s="5"/>
+    </row>
+    <row r="25" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1961,8 +2039,11 @@
       <c r="AW25" s="5"/>
       <c r="AX25" s="5"/>
       <c r="AY25" s="5"/>
-    </row>
-    <row r="26" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ25" s="5"/>
+      <c r="BA25" s="5"/>
+      <c r="BB25" s="5"/>
+    </row>
+    <row r="26" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -2014,8 +2095,11 @@
       <c r="AW26" s="5"/>
       <c r="AX26" s="5"/>
       <c r="AY26" s="5"/>
-    </row>
-    <row r="27" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ26" s="5"/>
+      <c r="BA26" s="5"/>
+      <c r="BB26" s="5"/>
+    </row>
+    <row r="27" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2067,8 +2151,11 @@
       <c r="AW27" s="5"/>
       <c r="AX27" s="5"/>
       <c r="AY27" s="5"/>
-    </row>
-    <row r="28" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ27" s="5"/>
+      <c r="BA27" s="5"/>
+      <c r="BB27" s="5"/>
+    </row>
+    <row r="28" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2120,8 +2207,11 @@
       <c r="AW28" s="5"/>
       <c r="AX28" s="5"/>
       <c r="AY28" s="5"/>
-    </row>
-    <row r="29" spans="1:51" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="AZ28" s="5"/>
+      <c r="BA28" s="5"/>
+      <c r="BB28" s="5"/>
+    </row>
+    <row r="29" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2173,12 +2263,15 @@
       <c r="AW29" s="5"/>
       <c r="AX29" s="5"/>
       <c r="AY29" s="5"/>
+      <c r="AZ29" s="5"/>
+      <c r="BA29" s="5"/>
+      <c r="BB29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AR5"/>
+    <mergeCell ref="A5:AU5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AR4"/>
+    <mergeCell ref="A4:AU4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
them cot si excel
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8F736E-6AF6-4FAB-A2A8-66CFF2EE5BBD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4F894D-F4CF-4686-8450-56362EC7D0A2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
   <si>
     <t>STT</t>
   </si>
@@ -164,6 +164,12 @@
   </si>
   <si>
     <t>KL gang CCT + Xỉ (T)</t>
+  </si>
+  <si>
+    <t>Nhiệt độ Gang</t>
+  </si>
+  <si>
+    <t>Si</t>
   </si>
 </sst>
 </file>
@@ -318,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -370,6 +376,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -729,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:BB29"/>
+  <dimension ref="A1:BD29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -740,41 +749,41 @@
     <col min="6" max="6" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" style="1" customWidth="1"/>
-    <col min="11" max="13" width="12.42578125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" style="1" customWidth="1"/>
-    <col min="15" max="16" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.85546875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="10.42578125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="16.85546875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="8.5703125" style="1" customWidth="1"/>
-    <col min="22" max="22" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="33.28515625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="14.7109375" style="1" customWidth="1"/>
-    <col min="26" max="26" width="12" style="1" customWidth="1"/>
-    <col min="27" max="27" width="9.7109375" style="1" customWidth="1"/>
-    <col min="28" max="30" width="9.42578125" style="1" customWidth="1"/>
-    <col min="31" max="31" width="12.42578125" style="1" customWidth="1"/>
-    <col min="32" max="32" width="10.42578125" style="1" customWidth="1"/>
-    <col min="33" max="33" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" style="1"/>
-    <col min="35" max="36" width="10.7109375" style="1" customWidth="1"/>
-    <col min="37" max="38" width="10.85546875" style="1" customWidth="1"/>
-    <col min="39" max="40" width="19.28515625" style="1" customWidth="1"/>
-    <col min="41" max="41" width="15.140625" style="1" customWidth="1"/>
-    <col min="42" max="42" width="12.28515625" style="1" customWidth="1"/>
-    <col min="43" max="43" width="13.140625" style="1" customWidth="1"/>
-    <col min="44" max="44" width="19.5703125" style="1" customWidth="1"/>
-    <col min="45" max="45" width="12.7109375" style="1" customWidth="1"/>
-    <col min="46" max="46" width="25.5703125" style="1" customWidth="1"/>
-    <col min="47" max="47" width="17.140625" style="1" customWidth="1"/>
-    <col min="48" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="11" width="9.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="19.85546875" style="1" customWidth="1"/>
+    <col min="13" max="15" width="12.42578125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.42578125" style="1" customWidth="1"/>
+    <col min="17" max="18" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="10.42578125" style="1" customWidth="1"/>
+    <col min="22" max="22" width="16.85546875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="8.5703125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="33.28515625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="14.7109375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="12" style="1" customWidth="1"/>
+    <col min="29" max="29" width="9.7109375" style="1" customWidth="1"/>
+    <col min="30" max="32" width="9.42578125" style="1" customWidth="1"/>
+    <col min="33" max="33" width="12.42578125" style="1" customWidth="1"/>
+    <col min="34" max="34" width="10.42578125" style="1" customWidth="1"/>
+    <col min="35" max="35" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="9.140625" style="1"/>
+    <col min="37" max="38" width="10.7109375" style="1" customWidth="1"/>
+    <col min="39" max="40" width="10.85546875" style="1" customWidth="1"/>
+    <col min="41" max="42" width="19.28515625" style="1" customWidth="1"/>
+    <col min="43" max="43" width="15.140625" style="1" customWidth="1"/>
+    <col min="44" max="44" width="12.28515625" style="1" customWidth="1"/>
+    <col min="45" max="45" width="13.140625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="19.5703125" style="1" customWidth="1"/>
+    <col min="47" max="47" width="12.7109375" style="1" customWidth="1"/>
+    <col min="48" max="48" width="25.5703125" style="1" customWidth="1"/>
+    <col min="49" max="49" width="17.140625" style="1" customWidth="1"/>
+    <col min="50" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:56" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -783,7 +792,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:54" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:56" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -792,7 +801,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:54" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:56" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -842,8 +851,10 @@
       <c r="AS4" s="19"/>
       <c r="AT4" s="19"/>
       <c r="AU4" s="19"/>
-    </row>
-    <row r="5" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="AV4" s="19"/>
+      <c r="AW4" s="19"/>
+    </row>
+    <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -891,8 +902,10 @@
       <c r="AS5" s="17"/>
       <c r="AT5" s="17"/>
       <c r="AU5" s="17"/>
-    </row>
-    <row r="7" spans="1:54" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AV5" s="17"/>
+      <c r="AW5" s="17"/>
+    </row>
+    <row r="7" spans="1:56" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -920,122 +933,128 @@
       <c r="I7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="J7" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="M7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="N7" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="O7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="S7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="T7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="S7" s="9" t="s">
+      <c r="U7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="T7" s="9" t="s">
+      <c r="V7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="U7" s="10" t="s">
+      <c r="W7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="V7" s="10" t="s">
+      <c r="X7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="W7" s="10" t="s">
+      <c r="Y7" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="X7" s="10" t="s">
+      <c r="Z7" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="Y7" s="10" t="s">
+      <c r="AA7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="Z7" s="10" t="s">
+      <c r="AB7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AA7" s="10" t="s">
+      <c r="AC7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AB7" s="10" t="s">
+      <c r="AD7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="AC7" s="10" t="s">
+      <c r="AE7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="AD7" s="10" t="s">
+      <c r="AF7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="AE7" s="10" t="s">
+      <c r="AG7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AH7" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="AG7" s="10" t="s">
+      <c r="AI7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="AH7" s="10" t="s">
+      <c r="AJ7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AI7" s="10" t="s">
+      <c r="AK7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="AJ7" s="10" t="s">
+      <c r="AL7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AK7" s="10" t="s">
+      <c r="AM7" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="AL7" s="10" t="s">
+      <c r="AN7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="AM7" s="10" t="s">
+      <c r="AO7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="AN7" s="10" t="s">
+      <c r="AP7" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="AO7" s="10" t="s">
+      <c r="AQ7" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="AP7" s="10" t="s">
+      <c r="AR7" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="AQ7" s="10" t="s">
+      <c r="AS7" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="AR7" s="11" t="s">
+      <c r="AT7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AS7" s="12" t="s">
+      <c r="AU7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="AT7" s="12" t="s">
+      <c r="AV7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="AU7" s="12" t="s">
+      <c r="AW7" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:56" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -1049,15 +1068,15 @@
       <c r="K8" s="14"/>
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
       <c r="P8" s="15"/>
       <c r="Q8" s="15"/>
-      <c r="R8" s="16"/>
+      <c r="R8" s="15"/>
       <c r="S8" s="15"/>
-      <c r="T8" s="15"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="13"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="15"/>
+      <c r="V8" s="15"/>
       <c r="W8" s="13"/>
       <c r="X8" s="13"/>
       <c r="Y8" s="13"/>
@@ -1079,19 +1098,21 @@
       <c r="AO8" s="13"/>
       <c r="AP8" s="13"/>
       <c r="AQ8" s="13"/>
-      <c r="AR8" s="15"/>
-      <c r="AS8" s="15"/>
+      <c r="AR8" s="13"/>
+      <c r="AS8" s="13"/>
       <c r="AT8" s="15"/>
       <c r="AU8" s="15"/>
-      <c r="AV8" s="5"/>
-      <c r="AW8" s="5"/>
+      <c r="AV8" s="15"/>
+      <c r="AW8" s="15"/>
       <c r="AX8" s="5"/>
       <c r="AY8" s="5"/>
       <c r="AZ8" s="5"/>
       <c r="BA8" s="5"/>
       <c r="BB8" s="5"/>
-    </row>
-    <row r="9" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BC8" s="5"/>
+      <c r="BD8" s="5"/>
+    </row>
+    <row r="9" spans="1:56" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1110,9 +1131,9 @@
       <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
       <c r="R9" s="6"/>
-      <c r="S9" s="7"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="7"/>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
       <c r="X9" s="5"/>
@@ -1146,8 +1167,10 @@
       <c r="AZ9" s="5"/>
       <c r="BA9" s="5"/>
       <c r="BB9" s="5"/>
-    </row>
-    <row r="10" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BC9" s="5"/>
+      <c r="BD9" s="5"/>
+    </row>
+    <row r="10" spans="1:56" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1166,9 +1189,9 @@
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
-      <c r="S10" s="7"/>
-      <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="7"/>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
       <c r="X10" s="5"/>
@@ -1202,8 +1225,10 @@
       <c r="AZ10" s="5"/>
       <c r="BA10" s="5"/>
       <c r="BB10" s="5"/>
-    </row>
-    <row r="11" spans="1:54" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BC10" s="5"/>
+      <c r="BD10" s="5"/>
+    </row>
+    <row r="11" spans="1:56" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1222,9 +1247,9 @@
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
       <c r="R11" s="6"/>
-      <c r="S11" s="7"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="7"/>
       <c r="V11" s="5"/>
       <c r="W11" s="5"/>
       <c r="X11" s="5"/>
@@ -1258,8 +1283,10 @@
       <c r="AZ11" s="5"/>
       <c r="BA11" s="5"/>
       <c r="BB11" s="5"/>
-    </row>
-    <row r="12" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC11" s="5"/>
+      <c r="BD11" s="5"/>
+    </row>
+    <row r="12" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1314,8 +1341,10 @@
       <c r="AZ12" s="5"/>
       <c r="BA12" s="5"/>
       <c r="BB12" s="5"/>
-    </row>
-    <row r="13" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC12" s="5"/>
+      <c r="BD12" s="5"/>
+    </row>
+    <row r="13" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -1370,8 +1399,10 @@
       <c r="AZ13" s="5"/>
       <c r="BA13" s="5"/>
       <c r="BB13" s="5"/>
-    </row>
-    <row r="14" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC13" s="5"/>
+      <c r="BD13" s="5"/>
+    </row>
+    <row r="14" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1426,8 +1457,10 @@
       <c r="AZ14" s="5"/>
       <c r="BA14" s="5"/>
       <c r="BB14" s="5"/>
-    </row>
-    <row r="15" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC14" s="5"/>
+      <c r="BD14" s="5"/>
+    </row>
+    <row r="15" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -1482,8 +1515,10 @@
       <c r="AZ15" s="5"/>
       <c r="BA15" s="5"/>
       <c r="BB15" s="5"/>
-    </row>
-    <row r="16" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC15" s="5"/>
+      <c r="BD15" s="5"/>
+    </row>
+    <row r="16" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1538,8 +1573,10 @@
       <c r="AZ16" s="5"/>
       <c r="BA16" s="5"/>
       <c r="BB16" s="5"/>
-    </row>
-    <row r="17" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC16" s="5"/>
+      <c r="BD16" s="5"/>
+    </row>
+    <row r="17" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1594,8 +1631,10 @@
       <c r="AZ17" s="5"/>
       <c r="BA17" s="5"/>
       <c r="BB17" s="5"/>
-    </row>
-    <row r="18" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC17" s="5"/>
+      <c r="BD17" s="5"/>
+    </row>
+    <row r="18" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1650,8 +1689,10 @@
       <c r="AZ18" s="5"/>
       <c r="BA18" s="5"/>
       <c r="BB18" s="5"/>
-    </row>
-    <row r="19" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC18" s="5"/>
+      <c r="BD18" s="5"/>
+    </row>
+    <row r="19" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -1706,8 +1747,10 @@
       <c r="AZ19" s="5"/>
       <c r="BA19" s="5"/>
       <c r="BB19" s="5"/>
-    </row>
-    <row r="20" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC19" s="5"/>
+      <c r="BD19" s="5"/>
+    </row>
+    <row r="20" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -1762,8 +1805,10 @@
       <c r="AZ20" s="5"/>
       <c r="BA20" s="5"/>
       <c r="BB20" s="5"/>
-    </row>
-    <row r="21" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC20" s="5"/>
+      <c r="BD20" s="5"/>
+    </row>
+    <row r="21" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1818,8 +1863,10 @@
       <c r="AZ21" s="5"/>
       <c r="BA21" s="5"/>
       <c r="BB21" s="5"/>
-    </row>
-    <row r="22" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC21" s="5"/>
+      <c r="BD21" s="5"/>
+    </row>
+    <row r="22" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1874,8 +1921,10 @@
       <c r="AZ22" s="5"/>
       <c r="BA22" s="5"/>
       <c r="BB22" s="5"/>
-    </row>
-    <row r="23" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC22" s="5"/>
+      <c r="BD22" s="5"/>
+    </row>
+    <row r="23" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1930,8 +1979,10 @@
       <c r="AZ23" s="5"/>
       <c r="BA23" s="5"/>
       <c r="BB23" s="5"/>
-    </row>
-    <row r="24" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC23" s="5"/>
+      <c r="BD23" s="5"/>
+    </row>
+    <row r="24" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1986,8 +2037,10 @@
       <c r="AZ24" s="5"/>
       <c r="BA24" s="5"/>
       <c r="BB24" s="5"/>
-    </row>
-    <row r="25" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC24" s="5"/>
+      <c r="BD24" s="5"/>
+    </row>
+    <row r="25" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -2042,8 +2095,10 @@
       <c r="AZ25" s="5"/>
       <c r="BA25" s="5"/>
       <c r="BB25" s="5"/>
-    </row>
-    <row r="26" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC25" s="5"/>
+      <c r="BD25" s="5"/>
+    </row>
+    <row r="26" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -2098,8 +2153,10 @@
       <c r="AZ26" s="5"/>
       <c r="BA26" s="5"/>
       <c r="BB26" s="5"/>
-    </row>
-    <row r="27" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC26" s="5"/>
+      <c r="BD26" s="5"/>
+    </row>
+    <row r="27" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2154,8 +2211,10 @@
       <c r="AZ27" s="5"/>
       <c r="BA27" s="5"/>
       <c r="BB27" s="5"/>
-    </row>
-    <row r="28" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC27" s="5"/>
+      <c r="BD27" s="5"/>
+    </row>
+    <row r="28" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2210,8 +2269,10 @@
       <c r="AZ28" s="5"/>
       <c r="BA28" s="5"/>
       <c r="BB28" s="5"/>
-    </row>
-    <row r="29" spans="1:54" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BC28" s="5"/>
+      <c r="BD28" s="5"/>
+    </row>
+    <row r="29" spans="1:56" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2266,12 +2327,14 @@
       <c r="AZ29" s="5"/>
       <c r="BA29" s="5"/>
       <c r="BB29" s="5"/>
+      <c r="BC29" s="5"/>
+      <c r="BD29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AU5"/>
+    <mergeCell ref="A5:AW5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AU4"/>
+    <mergeCell ref="A4:AW4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Chức năng xác nhận PL
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOFTWARE\DATA_PR\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A80B103C-3040-4057-A28D-E2C7D0651A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143E500C-E4F9-4811-B5D2-14F0A552D606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>STT</t>
   </si>
@@ -173,6 +173,9 @@
   </si>
   <si>
     <t>Phân loại LG TC04</t>
+  </si>
+  <si>
+    <t>Xác nhận không có mẫu TC06</t>
   </si>
 </sst>
 </file>
@@ -740,7 +743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:BE29"/>
+  <dimension ref="A1:BF29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -753,39 +756,39 @@
     <col min="8" max="8" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="11" width="9.42578125" style="1" customWidth="1"/>
     <col min="12" max="12" width="19.85546875" style="1" customWidth="1"/>
-    <col min="13" max="16" width="12.42578125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="9.42578125" style="1" customWidth="1"/>
-    <col min="18" max="19" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.85546875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="10.42578125" style="1" customWidth="1"/>
-    <col min="23" max="23" width="16.85546875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.5703125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="33.28515625" style="1" customWidth="1"/>
-    <col min="28" max="28" width="14.7109375" style="1" customWidth="1"/>
-    <col min="29" max="29" width="12" style="1" customWidth="1"/>
-    <col min="30" max="30" width="9.7109375" style="1" customWidth="1"/>
-    <col min="31" max="33" width="9.42578125" style="1" customWidth="1"/>
-    <col min="34" max="34" width="12.42578125" style="1" customWidth="1"/>
-    <col min="35" max="35" width="10.42578125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.140625" style="1"/>
-    <col min="38" max="39" width="10.7109375" style="1" customWidth="1"/>
-    <col min="40" max="41" width="10.85546875" style="1" customWidth="1"/>
-    <col min="42" max="43" width="19.28515625" style="1" customWidth="1"/>
-    <col min="44" max="44" width="15.140625" style="1" customWidth="1"/>
-    <col min="45" max="45" width="12.28515625" style="1" customWidth="1"/>
-    <col min="46" max="46" width="13.140625" style="1" customWidth="1"/>
-    <col min="47" max="47" width="19.5703125" style="1" customWidth="1"/>
-    <col min="48" max="48" width="12.7109375" style="1" customWidth="1"/>
-    <col min="49" max="49" width="25.5703125" style="1" customWidth="1"/>
-    <col min="50" max="50" width="17.140625" style="1" customWidth="1"/>
-    <col min="51" max="16384" width="9.140625" style="1"/>
+    <col min="13" max="17" width="12.42578125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="9.42578125" style="1" customWidth="1"/>
+    <col min="19" max="20" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="10.42578125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="16.85546875" style="1" customWidth="1"/>
+    <col min="25" max="25" width="8.5703125" style="1" customWidth="1"/>
+    <col min="26" max="26" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="33.28515625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="14.7109375" style="1" customWidth="1"/>
+    <col min="30" max="30" width="12" style="1" customWidth="1"/>
+    <col min="31" max="31" width="9.7109375" style="1" customWidth="1"/>
+    <col min="32" max="34" width="9.42578125" style="1" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="10.42578125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="9.140625" style="1"/>
+    <col min="39" max="40" width="10.7109375" style="1" customWidth="1"/>
+    <col min="41" max="42" width="10.85546875" style="1" customWidth="1"/>
+    <col min="43" max="44" width="19.28515625" style="1" customWidth="1"/>
+    <col min="45" max="45" width="15.140625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="12.28515625" style="1" customWidth="1"/>
+    <col min="47" max="47" width="13.140625" style="1" customWidth="1"/>
+    <col min="48" max="48" width="19.5703125" style="1" customWidth="1"/>
+    <col min="49" max="49" width="12.7109375" style="1" customWidth="1"/>
+    <col min="50" max="50" width="25.5703125" style="1" customWidth="1"/>
+    <col min="51" max="51" width="17.140625" style="1" customWidth="1"/>
+    <col min="52" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:58" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -794,7 +797,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:57" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -803,7 +806,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:57" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:58" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -856,8 +859,9 @@
       <c r="AV4" s="19"/>
       <c r="AW4" s="19"/>
       <c r="AX4" s="19"/>
-    </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
+      <c r="AY4" s="19"/>
+    </row>
+    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -908,8 +912,9 @@
       <c r="AV5" s="17"/>
       <c r="AW5" s="17"/>
       <c r="AX5" s="17"/>
-    </row>
-    <row r="7" spans="1:57" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AY5" s="17"/>
+    </row>
+    <row r="7" spans="1:58" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -952,116 +957,119 @@
       <c r="N7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="Q7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="S7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="S7" s="2" t="s">
+      <c r="T7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="U7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="U7" s="2" t="s">
+      <c r="V7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="V7" s="8" t="s">
+      <c r="W7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="W7" s="8" t="s">
+      <c r="X7" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="X7" s="9" t="s">
+      <c r="Y7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="Y7" s="9" t="s">
+      <c r="Z7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="Z7" s="9" t="s">
+      <c r="AA7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="AA7" s="9" t="s">
+      <c r="AB7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="AB7" s="9" t="s">
+      <c r="AC7" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="AC7" s="9" t="s">
+      <c r="AD7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AD7" s="9" t="s">
+      <c r="AE7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AE7" s="9" t="s">
+      <c r="AF7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AF7" s="9" t="s">
+      <c r="AG7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="AG7" s="9" t="s">
+      <c r="AH7" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="AH7" s="9" t="s">
+      <c r="AI7" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="AI7" s="9" t="s">
+      <c r="AJ7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AJ7" s="9" t="s">
+      <c r="AK7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="AK7" s="9" t="s">
+      <c r="AL7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="AL7" s="9" t="s">
+      <c r="AM7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AM7" s="9" t="s">
+      <c r="AN7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AN7" s="9" t="s">
+      <c r="AO7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AO7" s="9" t="s">
+      <c r="AP7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="AP7" s="9" t="s">
+      <c r="AQ7" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="AQ7" s="9" t="s">
+      <c r="AR7" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="AR7" s="9" t="s">
+      <c r="AS7" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="AS7" s="9" t="s">
+      <c r="AT7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="AT7" s="9" t="s">
+      <c r="AU7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="AU7" s="10" t="s">
+      <c r="AV7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="AV7" s="11" t="s">
+      <c r="AW7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AW7" s="11" t="s">
+      <c r="AX7" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="AX7" s="11" t="s">
+      <c r="AY7" s="11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:57" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:58" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -1078,14 +1086,14 @@
       <c r="N8" s="13"/>
       <c r="O8" s="13"/>
       <c r="P8" s="13"/>
-      <c r="Q8" s="14"/>
+      <c r="Q8" s="13"/>
       <c r="R8" s="14"/>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
-      <c r="U8" s="15"/>
-      <c r="V8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="15"/>
       <c r="W8" s="14"/>
-      <c r="X8" s="12"/>
+      <c r="X8" s="14"/>
       <c r="Y8" s="12"/>
       <c r="Z8" s="12"/>
       <c r="AA8" s="12"/>
@@ -1108,19 +1116,20 @@
       <c r="AR8" s="12"/>
       <c r="AS8" s="12"/>
       <c r="AT8" s="12"/>
-      <c r="AU8" s="14"/>
+      <c r="AU8" s="12"/>
       <c r="AV8" s="14"/>
       <c r="AW8" s="14"/>
       <c r="AX8" s="14"/>
-      <c r="AY8" s="4"/>
+      <c r="AY8" s="14"/>
       <c r="AZ8" s="4"/>
       <c r="BA8" s="4"/>
       <c r="BB8" s="4"/>
       <c r="BC8" s="4"/>
       <c r="BD8" s="4"/>
       <c r="BE8" s="4"/>
-    </row>
-    <row r="9" spans="1:57" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BF8" s="4"/>
+    </row>
+    <row r="9" spans="1:58" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1142,8 +1151,8 @@
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="4"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="6"/>
       <c r="X9" s="4"/>
       <c r="Y9" s="4"/>
       <c r="Z9" s="4"/>
@@ -1178,8 +1187,9 @@
       <c r="BC9" s="4"/>
       <c r="BD9" s="4"/>
       <c r="BE9" s="4"/>
-    </row>
-    <row r="10" spans="1:57" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BF9" s="4"/>
+    </row>
+    <row r="10" spans="1:58" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1201,8 +1211,8 @@
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="4"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="6"/>
       <c r="X10" s="4"/>
       <c r="Y10" s="4"/>
       <c r="Z10" s="4"/>
@@ -1237,8 +1247,9 @@
       <c r="BC10" s="4"/>
       <c r="BD10" s="4"/>
       <c r="BE10" s="4"/>
-    </row>
-    <row r="11" spans="1:57" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BF10" s="4"/>
+    </row>
+    <row r="11" spans="1:58" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1260,8 +1271,8 @@
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="4"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="6"/>
       <c r="X11" s="4"/>
       <c r="Y11" s="4"/>
       <c r="Z11" s="4"/>
@@ -1296,8 +1307,9 @@
       <c r="BC11" s="4"/>
       <c r="BD11" s="4"/>
       <c r="BE11" s="4"/>
-    </row>
-    <row r="12" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF11" s="4"/>
+    </row>
+    <row r="12" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1355,8 +1367,9 @@
       <c r="BC12" s="4"/>
       <c r="BD12" s="4"/>
       <c r="BE12" s="4"/>
-    </row>
-    <row r="13" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF12" s="4"/>
+    </row>
+    <row r="13" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1414,8 +1427,9 @@
       <c r="BC13" s="4"/>
       <c r="BD13" s="4"/>
       <c r="BE13" s="4"/>
-    </row>
-    <row r="14" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF13" s="4"/>
+    </row>
+    <row r="14" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1473,8 +1487,9 @@
       <c r="BC14" s="4"/>
       <c r="BD14" s="4"/>
       <c r="BE14" s="4"/>
-    </row>
-    <row r="15" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF14" s="4"/>
+    </row>
+    <row r="15" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1532,8 +1547,9 @@
       <c r="BC15" s="4"/>
       <c r="BD15" s="4"/>
       <c r="BE15" s="4"/>
-    </row>
-    <row r="16" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF15" s="4"/>
+    </row>
+    <row r="16" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1591,8 +1607,9 @@
       <c r="BC16" s="4"/>
       <c r="BD16" s="4"/>
       <c r="BE16" s="4"/>
-    </row>
-    <row r="17" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF16" s="4"/>
+    </row>
+    <row r="17" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1650,8 +1667,9 @@
       <c r="BC17" s="4"/>
       <c r="BD17" s="4"/>
       <c r="BE17" s="4"/>
-    </row>
-    <row r="18" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF17" s="4"/>
+    </row>
+    <row r="18" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1709,8 +1727,9 @@
       <c r="BC18" s="4"/>
       <c r="BD18" s="4"/>
       <c r="BE18" s="4"/>
-    </row>
-    <row r="19" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF18" s="4"/>
+    </row>
+    <row r="19" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1768,8 +1787,9 @@
       <c r="BC19" s="4"/>
       <c r="BD19" s="4"/>
       <c r="BE19" s="4"/>
-    </row>
-    <row r="20" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF19" s="4"/>
+    </row>
+    <row r="20" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1827,8 +1847,9 @@
       <c r="BC20" s="4"/>
       <c r="BD20" s="4"/>
       <c r="BE20" s="4"/>
-    </row>
-    <row r="21" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF20" s="4"/>
+    </row>
+    <row r="21" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1886,8 +1907,9 @@
       <c r="BC21" s="4"/>
       <c r="BD21" s="4"/>
       <c r="BE21" s="4"/>
-    </row>
-    <row r="22" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF21" s="4"/>
+    </row>
+    <row r="22" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1945,8 +1967,9 @@
       <c r="BC22" s="4"/>
       <c r="BD22" s="4"/>
       <c r="BE22" s="4"/>
-    </row>
-    <row r="23" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF22" s="4"/>
+    </row>
+    <row r="23" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -2004,8 +2027,9 @@
       <c r="BC23" s="4"/>
       <c r="BD23" s="4"/>
       <c r="BE23" s="4"/>
-    </row>
-    <row r="24" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF23" s="4"/>
+    </row>
+    <row r="24" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -2063,8 +2087,9 @@
       <c r="BC24" s="4"/>
       <c r="BD24" s="4"/>
       <c r="BE24" s="4"/>
-    </row>
-    <row r="25" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF24" s="4"/>
+    </row>
+    <row r="25" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2122,8 +2147,9 @@
       <c r="BC25" s="4"/>
       <c r="BD25" s="4"/>
       <c r="BE25" s="4"/>
-    </row>
-    <row r="26" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF25" s="4"/>
+    </row>
+    <row r="26" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2181,8 +2207,9 @@
       <c r="BC26" s="4"/>
       <c r="BD26" s="4"/>
       <c r="BE26" s="4"/>
-    </row>
-    <row r="27" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF26" s="4"/>
+    </row>
+    <row r="27" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -2240,8 +2267,9 @@
       <c r="BC27" s="4"/>
       <c r="BD27" s="4"/>
       <c r="BE27" s="4"/>
-    </row>
-    <row r="28" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF27" s="4"/>
+    </row>
+    <row r="28" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2299,8 +2327,9 @@
       <c r="BC28" s="4"/>
       <c r="BD28" s="4"/>
       <c r="BE28" s="4"/>
-    </row>
-    <row r="29" spans="1:57" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BF28" s="4"/>
+    </row>
+    <row r="29" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2358,12 +2387,13 @@
       <c r="BC29" s="4"/>
       <c r="BD29" s="4"/>
       <c r="BE29" s="4"/>
+      <c r="BF29" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AX5"/>
+    <mergeCell ref="A5:AY5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AX4"/>
+    <mergeCell ref="A4:AY4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
thêm cột nhiệt độ export excel
</commit_message>
<xml_diff>
--- a/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
+++ b/Data_Product/App_Data/QTGN_Gang_Long_PKH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SOFTWARE\DATA_PR\Data_Product\App_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\DATAPRODUCT\DATAPRODUCT\Data_Product\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBC8F7D-EB29-4AE0-88C7-DC7BBF18CEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7495BFA-212A-497F-B93B-AE894AB635D9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{51577134-7CEF-4490-9A02-725D1462A1F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>STT</t>
   </si>
@@ -179,6 +179,9 @@
   </si>
   <si>
     <t>Phân loại LG TC06</t>
+  </si>
+  <si>
+    <t>Nhiệt độ Gang vào HRC</t>
   </si>
 </sst>
 </file>
@@ -746,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC901D94-D8FD-44B6-9D08-9B52821867A9}">
-  <dimension ref="A1:BF29"/>
+  <dimension ref="A1:BG29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
@@ -770,28 +773,28 @@
     <col min="26" max="26" width="7" style="1" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="33.28515625" style="1" customWidth="1"/>
-    <col min="29" max="29" width="14.7109375" style="1" customWidth="1"/>
-    <col min="30" max="30" width="12" style="1" customWidth="1"/>
-    <col min="31" max="31" width="9.7109375" style="1" customWidth="1"/>
-    <col min="32" max="34" width="9.42578125" style="1" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="10.42578125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="9.140625" style="1"/>
-    <col min="39" max="40" width="10.7109375" style="1" customWidth="1"/>
-    <col min="41" max="42" width="10.85546875" style="1" customWidth="1"/>
-    <col min="43" max="44" width="19.28515625" style="1" customWidth="1"/>
-    <col min="45" max="45" width="15.140625" style="1" customWidth="1"/>
-    <col min="46" max="46" width="12.28515625" style="1" customWidth="1"/>
-    <col min="47" max="47" width="13.140625" style="1" customWidth="1"/>
-    <col min="48" max="48" width="19.5703125" style="1" customWidth="1"/>
-    <col min="49" max="49" width="12.7109375" style="1" customWidth="1"/>
-    <col min="50" max="50" width="25.5703125" style="1" customWidth="1"/>
-    <col min="51" max="51" width="17.140625" style="1" customWidth="1"/>
-    <col min="52" max="16384" width="9.140625" style="1"/>
+    <col min="29" max="30" width="14.7109375" style="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="1" customWidth="1"/>
+    <col min="32" max="32" width="9.7109375" style="1" customWidth="1"/>
+    <col min="33" max="35" width="9.42578125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="12.42578125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="10.42578125" style="1" customWidth="1"/>
+    <col min="38" max="38" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="9.140625" style="1"/>
+    <col min="40" max="41" width="10.7109375" style="1" customWidth="1"/>
+    <col min="42" max="43" width="10.85546875" style="1" customWidth="1"/>
+    <col min="44" max="45" width="19.28515625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="15.140625" style="1" customWidth="1"/>
+    <col min="47" max="47" width="12.28515625" style="1" customWidth="1"/>
+    <col min="48" max="48" width="13.140625" style="1" customWidth="1"/>
+    <col min="49" max="49" width="19.5703125" style="1" customWidth="1"/>
+    <col min="50" max="50" width="12.7109375" style="1" customWidth="1"/>
+    <col min="51" max="51" width="25.5703125" style="1" customWidth="1"/>
+    <col min="52" max="52" width="17.140625" style="1" customWidth="1"/>
+    <col min="53" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:58" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:59" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
@@ -800,7 +803,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
     </row>
-    <row r="2" spans="1:58" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:59" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -809,7 +812,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="18"/>
     </row>
-    <row r="4" spans="1:58" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:59" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>8</v>
       </c>
@@ -863,8 +866,9 @@
       <c r="AW4" s="19"/>
       <c r="AX4" s="19"/>
       <c r="AY4" s="19"/>
-    </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="AZ4" s="19"/>
+    </row>
+    <row r="5" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -916,8 +920,9 @@
       <c r="AW5" s="17"/>
       <c r="AX5" s="17"/>
       <c r="AY5" s="17"/>
-    </row>
-    <row r="7" spans="1:58" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AZ5" s="17"/>
+    </row>
+    <row r="7" spans="1:59" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
@@ -1006,76 +1011,79 @@
         <v>1</v>
       </c>
       <c r="AD7" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE7" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="AE7" s="9" t="s">
+      <c r="AF7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AF7" s="9" t="s">
+      <c r="AG7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AG7" s="9" t="s">
+      <c r="AH7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AH7" s="9" t="s">
+      <c r="AI7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="AI7" s="9" t="s">
+      <c r="AJ7" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="AJ7" s="9" t="s">
+      <c r="AK7" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="AK7" s="9" t="s">
+      <c r="AL7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AL7" s="9" t="s">
+      <c r="AM7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="AM7" s="9" t="s">
+      <c r="AN7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="AN7" s="9" t="s">
+      <c r="AO7" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="AO7" s="9" t="s">
+      <c r="AP7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="AP7" s="9" t="s">
+      <c r="AQ7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AQ7" s="9" t="s">
+      <c r="AR7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="AR7" s="9" t="s">
+      <c r="AS7" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="AS7" s="9" t="s">
+      <c r="AT7" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="AT7" s="9" t="s">
+      <c r="AU7" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="AU7" s="9" t="s">
+      <c r="AV7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="AV7" s="9" t="s">
+      <c r="AW7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="AW7" s="10" t="s">
+      <c r="AX7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="AX7" s="11" t="s">
+      <c r="AY7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="AY7" s="11" t="s">
+      <c r="AZ7" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="AZ7" s="11" t="s">
+      <c r="BA7" s="11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:58" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:59" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -1123,19 +1131,20 @@
       <c r="AS8" s="12"/>
       <c r="AT8" s="12"/>
       <c r="AU8" s="12"/>
-      <c r="AV8" s="14"/>
+      <c r="AV8" s="12"/>
       <c r="AW8" s="14"/>
       <c r="AX8" s="14"/>
       <c r="AY8" s="14"/>
-      <c r="AZ8" s="4"/>
+      <c r="AZ8" s="14"/>
       <c r="BA8" s="4"/>
       <c r="BB8" s="4"/>
       <c r="BC8" s="4"/>
       <c r="BD8" s="4"/>
       <c r="BE8" s="4"/>
       <c r="BF8" s="4"/>
-    </row>
-    <row r="9" spans="1:58" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BG8" s="4"/>
+    </row>
+    <row r="9" spans="1:59" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -1194,8 +1203,9 @@
       <c r="BD9" s="4"/>
       <c r="BE9" s="4"/>
       <c r="BF9" s="4"/>
-    </row>
-    <row r="10" spans="1:58" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BG9" s="4"/>
+    </row>
+    <row r="10" spans="1:59" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1254,8 +1264,9 @@
       <c r="BD10" s="4"/>
       <c r="BE10" s="4"/>
       <c r="BF10" s="4"/>
-    </row>
-    <row r="11" spans="1:58" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="BG10" s="4"/>
+    </row>
+    <row r="11" spans="1:59" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -1314,8 +1325,9 @@
       <c r="BD11" s="4"/>
       <c r="BE11" s="4"/>
       <c r="BF11" s="4"/>
-    </row>
-    <row r="12" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG11" s="4"/>
+    </row>
+    <row r="12" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1374,8 +1386,9 @@
       <c r="BD12" s="4"/>
       <c r="BE12" s="4"/>
       <c r="BF12" s="4"/>
-    </row>
-    <row r="13" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG12" s="4"/>
+    </row>
+    <row r="13" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1434,8 +1447,9 @@
       <c r="BD13" s="4"/>
       <c r="BE13" s="4"/>
       <c r="BF13" s="4"/>
-    </row>
-    <row r="14" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG13" s="4"/>
+    </row>
+    <row r="14" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1494,8 +1508,9 @@
       <c r="BD14" s="4"/>
       <c r="BE14" s="4"/>
       <c r="BF14" s="4"/>
-    </row>
-    <row r="15" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG14" s="4"/>
+    </row>
+    <row r="15" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1554,8 +1569,9 @@
       <c r="BD15" s="4"/>
       <c r="BE15" s="4"/>
       <c r="BF15" s="4"/>
-    </row>
-    <row r="16" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG15" s="4"/>
+    </row>
+    <row r="16" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -1614,8 +1630,9 @@
       <c r="BD16" s="4"/>
       <c r="BE16" s="4"/>
       <c r="BF16" s="4"/>
-    </row>
-    <row r="17" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG16" s="4"/>
+    </row>
+    <row r="17" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1674,8 +1691,9 @@
       <c r="BD17" s="4"/>
       <c r="BE17" s="4"/>
       <c r="BF17" s="4"/>
-    </row>
-    <row r="18" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG17" s="4"/>
+    </row>
+    <row r="18" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1734,8 +1752,9 @@
       <c r="BD18" s="4"/>
       <c r="BE18" s="4"/>
       <c r="BF18" s="4"/>
-    </row>
-    <row r="19" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG18" s="4"/>
+    </row>
+    <row r="19" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -1794,8 +1813,9 @@
       <c r="BD19" s="4"/>
       <c r="BE19" s="4"/>
       <c r="BF19" s="4"/>
-    </row>
-    <row r="20" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG19" s="4"/>
+    </row>
+    <row r="20" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1854,8 +1874,9 @@
       <c r="BD20" s="4"/>
       <c r="BE20" s="4"/>
       <c r="BF20" s="4"/>
-    </row>
-    <row r="21" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG20" s="4"/>
+    </row>
+    <row r="21" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -1914,8 +1935,9 @@
       <c r="BD21" s="4"/>
       <c r="BE21" s="4"/>
       <c r="BF21" s="4"/>
-    </row>
-    <row r="22" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG21" s="4"/>
+    </row>
+    <row r="22" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -1974,8 +1996,9 @@
       <c r="BD22" s="4"/>
       <c r="BE22" s="4"/>
       <c r="BF22" s="4"/>
-    </row>
-    <row r="23" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG22" s="4"/>
+    </row>
+    <row r="23" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
@@ -2034,8 +2057,9 @@
       <c r="BD23" s="4"/>
       <c r="BE23" s="4"/>
       <c r="BF23" s="4"/>
-    </row>
-    <row r="24" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG23" s="4"/>
+    </row>
+    <row r="24" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -2094,8 +2118,9 @@
       <c r="BD24" s="4"/>
       <c r="BE24" s="4"/>
       <c r="BF24" s="4"/>
-    </row>
-    <row r="25" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG24" s="4"/>
+    </row>
+    <row r="25" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
@@ -2154,8 +2179,9 @@
       <c r="BD25" s="4"/>
       <c r="BE25" s="4"/>
       <c r="BF25" s="4"/>
-    </row>
-    <row r="26" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG25" s="4"/>
+    </row>
+    <row r="26" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2214,8 +2240,9 @@
       <c r="BD26" s="4"/>
       <c r="BE26" s="4"/>
       <c r="BF26" s="4"/>
-    </row>
-    <row r="27" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG26" s="4"/>
+    </row>
+    <row r="27" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -2274,8 +2301,9 @@
       <c r="BD27" s="4"/>
       <c r="BE27" s="4"/>
       <c r="BF27" s="4"/>
-    </row>
-    <row r="28" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG27" s="4"/>
+    </row>
+    <row r="28" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2334,8 +2362,9 @@
       <c r="BD28" s="4"/>
       <c r="BE28" s="4"/>
       <c r="BF28" s="4"/>
-    </row>
-    <row r="29" spans="1:58" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="BG28" s="4"/>
+    </row>
+    <row r="29" spans="1:59" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2394,12 +2423,13 @@
       <c r="BD29" s="4"/>
       <c r="BE29" s="4"/>
       <c r="BF29" s="4"/>
+      <c r="BG29" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A5:AY5"/>
+    <mergeCell ref="A5:AZ5"/>
     <mergeCell ref="B1:H2"/>
-    <mergeCell ref="A4:AY4"/>
+    <mergeCell ref="A4:AZ4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>